<commit_message>
Red-team fixes and PDF user manuals (FR/EN) for all three products
- Model fix: battery round-trip efficiency added to P1 and P2; night-time solar
  energy now carries the storage loss in sizing and in solar delivery
- Financing request wording fixed (no article before the generator size)
- Six PDF manuals (three products, French and English) built from Markdown with
  WeasyPrint: cover, paginated contents, running heads, French typography
- Manual build checks: no em/en dashes, no stock phrases, and every quoted label
  must exist in the matching workbook (cells, sheet names or formula literals)
- Markdown quick guides replaced by the manuals; listings and figures updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BXecWCCHxS2NDKTkshp3of
</commit_message>
<xml_diff>
--- a/product/03-fund-manager/EnergyAccess_Fund_Manager_Model_v1.xlsx
+++ b/product/03-fund-manager/EnergyAccess_Fund_Manager_Model_v1.xlsx
@@ -1863,11 +1863,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="6888949"/>
-        <c:axId val="79189285"/>
+        <c:axId val="91920957"/>
+        <c:axId val="95426669"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="6888949"/>
+        <c:axId val="91920957"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1899,7 +1899,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79189285"/>
+        <c:crossAx val="95426669"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1907,7 +1907,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79189285"/>
+        <c:axId val="95426669"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1949,7 +1949,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6888949"/>
+        <c:crossAx val="91920957"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2276,8 +2276,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="37079715"/>
-        <c:axId val="94626640"/>
+        <c:axId val="81564666"/>
+        <c:axId val="68640032"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -2422,11 +2422,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="53709899"/>
-        <c:axId val="41767801"/>
+        <c:axId val="35460353"/>
+        <c:axId val="31291177"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="37079715"/>
+        <c:axId val="81564666"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2458,7 +2458,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94626640"/>
+        <c:crossAx val="68640032"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2466,7 +2466,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94626640"/>
+        <c:axId val="68640032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2508,12 +2508,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37079715"/>
+        <c:crossAx val="81564666"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="53709899"/>
+        <c:axId val="35460353"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2545,7 +2545,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="41767801"/>
+        <c:crossAx val="31291177"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2553,7 +2553,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="41767801"/>
+        <c:axId val="31291177"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2619,7 +2619,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53709899"/>
+        <c:crossAx val="35460353"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
P3 example: set over-commitment ratio to 1.00
- Example fund now commits exactly the available funds; all four portfolio verdicts pass
- P3 manuals (FR/EN): worked example updated with recalculated figures; the 1.10 case
  is kept as an explicit what-if showing why over-commitment fails with a grant-heavy mix
- P3 workbooks (EN/FR) and listing images regenerated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BXecWCCHxS2NDKTkshp3of
</commit_message>
<xml_diff>
--- a/product/03-fund-manager/EnergyAccess_Fund_Manager_Model_v1.xlsx
+++ b/product/03-fund-manager/EnergyAccess_Fund_Manager_Model_v1.xlsx
@@ -1777,10 +1777,10 @@
                   <c:v>Project N - Lakeside expansion</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>Project B - River towns</c:v>
+                  <c:v>Project I - Fishing communities</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Project I - Fishing communities</c:v>
+                  <c:v>Project B - River towns</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v/>
@@ -1813,28 +1813,28 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="15"/>
                 <c:pt idx="0">
-                  <c:v>420750</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>420750</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>420750</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>420750</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>420750</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>140250</c:v>
+                  <c:v>127500</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>320000</c:v>
+                  <c:v>382500</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>241000</c:v>
+                  <c:v>127500</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -1863,11 +1863,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="91920957"/>
-        <c:axId val="95426669"/>
+        <c:axId val="35660604"/>
+        <c:axId val="90834697"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="91920957"/>
+        <c:axId val="35660604"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1899,7 +1899,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95426669"/>
+        <c:crossAx val="90834697"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1907,7 +1907,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95426669"/>
+        <c:axId val="90834697"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1949,7 +1949,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="91920957"/>
+        <c:crossAx val="35660604"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2115,19 +2115,19 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>156598.271110424</c:v>
+                  <c:v>142362.06464584</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>314245.030447853</c:v>
+                  <c:v>287482.814784728</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>216429.380782786</c:v>
+                  <c:v>198430.531594709</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>75502.676557804</c:v>
+                  <c:v>69326.6118717172</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>12059.4535807879</c:v>
+                  <c:v>11092.1049315831</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>0</c:v>
@@ -2241,10 +2241,10 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>876442.858615763</c:v>
+                  <c:v>796766.235105239</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1105169.38000596</c:v>
+                  <c:v>999922.943306651</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2276,8 +2276,8 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="81564666"/>
-        <c:axId val="68640032"/>
+        <c:axId val="46613232"/>
+        <c:axId val="93878166"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -2380,34 +2380,34 @@
                 <c:formatCode>#,##0;\(#,##0\);\-</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>1033041.12972619</c:v>
+                  <c:v>939128.299751079</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2452455.54018</c:v>
+                  <c:v>2226534.05784246</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2668884.92096279</c:v>
+                  <c:v>2424964.58943717</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2744387.59752059</c:v>
+                  <c:v>2494291.20130888</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2756447.05110138</c:v>
+                  <c:v>2505383.30624047</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2422,11 +2422,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="35460353"/>
-        <c:axId val="31291177"/>
+        <c:axId val="92978840"/>
+        <c:axId val="41002277"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="81564666"/>
+        <c:axId val="46613232"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2458,7 +2458,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="68640032"/>
+        <c:crossAx val="93878166"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2466,7 +2466,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="68640032"/>
+        <c:axId val="93878166"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2508,12 +2508,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81564666"/>
+        <c:crossAx val="46613232"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="35460353"/>
+        <c:axId val="92978840"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2545,7 +2545,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31291177"/>
+        <c:crossAx val="41002277"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2553,7 +2553,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31291177"/>
+        <c:axId val="41002277"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2619,7 +2619,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35460353"/>
+        <c:crossAx val="92978840"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3117,16 +3117,16 @@
                 <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>740750</c:v>
+                  <c:v>510000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1402500</c:v>
+                  <c:v>1275000</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>661750</c:v>
+                  <c:v>765000</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -3760,7 +3760,7 @@
         <v>45</v>
       </c>
       <c r="B13" s="17" t="n">
-        <v>1.1</v>
+        <v>1</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>46</v>
@@ -3772,7 +3772,7 @@
       </c>
       <c r="B14" s="16" t="n">
         <f aca="false">Available*Overcommit</f>
-        <v>2805000</v>
+        <v>2550000</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6027,11 +6027,11 @@
       </c>
       <c r="S7" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q7+$R7,MaxSupportPct*Pipeline!$N7-Pipeline!$Q7,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T7" s="28" t="n">
         <f aca="false">IF($O7=1,IF(Pipeline!$V7&gt;0,MIN(Pipeline!$V7,$S7),$S7),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U7" s="29" t="n">
         <f aca="false">IFERROR($Q7/($Q7+$R7),1)</f>
@@ -6039,15 +6039,15 @@
       </c>
       <c r="V7" s="28" t="n">
         <f aca="false">IFERROR($T7/$C7,0)</f>
-        <v>389.583333333333</v>
+        <v>354.166666666667</v>
       </c>
       <c r="W7" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O7+Pipeline!$P7)/$T7,0)</f>
-        <v>1.30718954248366</v>
+        <v>1.43790849673203</v>
       </c>
       <c r="X7" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T7/$T7*1000,0)</f>
-        <v>16.6369578134284</v>
+        <v>18.3006535947712</v>
       </c>
       <c r="Y7" s="30" t="str">
         <f aca="false">IF($O7=0,"",IF(NOT(ISNUMBER(Pipeline!$U7)),"No viability-gap data",IF(Pipeline!$U7&lt;=0,"No viability-gap data",IF($T7&lt;=Pipeline!$U7*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="AK7" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,1,Allocation!$I$7:$I$31)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="AL7" s="29" t="n">
         <f aca="false">IFERROR($AK7/$T7,0)</f>
@@ -6111,11 +6111,11 @@
       </c>
       <c r="AN7" s="37" t="n">
         <f aca="false">IF(AND($O7=1,$V7&gt;0),1/$V7,0)</f>
-        <v>0.0025668449197861</v>
+        <v>0.00282352941176471</v>
       </c>
       <c r="AO7" s="38" t="n">
         <f aca="false">IF($O7=1,$W7,0)</f>
-        <v>1.30718954248366</v>
+        <v>1.43790849673203</v>
       </c>
       <c r="AP7" s="39" t="n">
         <f aca="false">IF($O7=1,$F7,0)</f>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="AQ7" s="37" t="n">
         <f aca="false">IF(AND($O7=1,$T7&gt;0),Pipeline!$T7/$T7,0)</f>
-        <v>0.0166369578134284</v>
+        <v>0.0183006535947712</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6229,11 +6229,11 @@
       </c>
       <c r="Z8" s="33" t="n">
         <f aca="false">IF($O8=1,IFERROR($AN8/MAX($AN$7:$AN$31)*100,0),0)</f>
-        <v>53.3915548424738</v>
+        <v>48.5377771295216</v>
       </c>
       <c r="AA8" s="33" t="n">
         <f aca="false">IF($O8=1,IFERROR($AO8/MAX($AO$7:$AO$31)*100,0),0)</f>
-        <v>46.01953125</v>
+        <v>41.8359375</v>
       </c>
       <c r="AB8" s="33" t="n">
         <f aca="false">IF($O8=1,IFERROR($AP8/MAX($AP$7:$AP$31)*100,0),0)</f>
@@ -6241,7 +6241,7 @@
       </c>
       <c r="AC8" s="33" t="n">
         <f aca="false">IF($O8=1,IFERROR($AQ8/MAX($AQ$7:$AQ$31)*100,0),0)</f>
-        <v>49.306640625</v>
+        <v>44.82421875</v>
       </c>
       <c r="AD8" s="33" t="n">
         <f aca="false">IF($O8=1,Pipeline!$F8/5*100,0)</f>
@@ -6261,27 +6261,27 @@
       </c>
       <c r="AH8" s="34" t="n">
         <f aca="false">$Z8*W_Cost+$AA8*W_Lev+$AB8*W_PU+$AC8*W_CO2+$AD8*W_Ready+$AE8*W_Track+$AF8*W_Risk+$AG8*W_Add</f>
-        <v>54.2270489630815</v>
+        <v>51.9378232848435</v>
       </c>
       <c r="AI8" s="35" t="n">
         <f aca="false">IF($O8=1,$AH8+(26-$A8)/1000000,-1)</f>
-        <v>54.2270729630815</v>
+        <v>51.9378472848435</v>
       </c>
       <c r="AJ8" s="21" t="n">
         <f aca="false">IF($O8=1,COUNTIF($AI$7:$AI$31,"&gt;"&amp;$AI8)+1,"")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AK8" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,2,Allocation!$I$7:$I$31)</f>
-        <v>320000</v>
+        <v>127500</v>
       </c>
       <c r="AL8" s="29" t="n">
         <f aca="false">IFERROR($AK8/$T8,0)</f>
-        <v>1</v>
+        <v>0.3984375</v>
       </c>
       <c r="AM8" s="30" t="str">
         <f aca="false">IF($O8=0,"",IF($AL8&gt;=0.999,"Funded",IF($AK8&gt;0,"Partially funded","Not funded")))</f>
-        <v>Funded</v>
+        <v>Partially funded</v>
       </c>
       <c r="AN8" s="37" t="n">
         <f aca="false">IF(AND($O8=1,$V8&gt;0),1/$V8,0)</f>
@@ -6375,11 +6375,11 @@
       </c>
       <c r="S9" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q9+$R9,MaxSupportPct*Pipeline!$N9-Pipeline!$Q9,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T9" s="28" t="n">
         <f aca="false">IF($O9=1,IF(Pipeline!$V9&gt;0,MIN(Pipeline!$V9,$S9),$S9),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U9" s="29" t="n">
         <f aca="false">IFERROR($Q9/($Q9+$R9),1)</f>
@@ -6387,15 +6387,15 @@
       </c>
       <c r="V9" s="28" t="n">
         <f aca="false">IFERROR($T9/$C9,0)</f>
-        <v>245.478413068845</v>
+        <v>223.16219369895</v>
       </c>
       <c r="W9" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O9+Pipeline!$P9)/$T9,0)</f>
-        <v>2.3767082590612</v>
+        <v>2.61437908496732</v>
       </c>
       <c r="X9" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T9/$T9*1000,0)</f>
-        <v>28.5204991087344</v>
+        <v>31.3725490196078</v>
       </c>
       <c r="Y9" s="30" t="str">
         <f aca="false">IF($O9=0,"",IF(NOT(ISNUMBER(Pipeline!$U9)),"No viability-gap data",IF(Pipeline!$U9&lt;=0,"No viability-gap data",IF($T9&lt;=Pipeline!$U9*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="AK9" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,3,Allocation!$I$7:$I$31)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="AL9" s="29" t="n">
         <f aca="false">IFERROR($AK9/$T9,0)</f>
@@ -6459,11 +6459,11 @@
       </c>
       <c r="AN9" s="37" t="n">
         <f aca="false">IF(AND($O9=1,$V9&gt;0),1/$V9,0)</f>
-        <v>0.0040736779560309</v>
+        <v>0.00448104575163399</v>
       </c>
       <c r="AO9" s="38" t="n">
         <f aca="false">IF($O9=1,$W9,0)</f>
-        <v>2.3767082590612</v>
+        <v>2.61437908496732</v>
       </c>
       <c r="AP9" s="39" t="n">
         <f aca="false">IF($O9=1,$F9,0)</f>
@@ -6471,7 +6471,7 @@
       </c>
       <c r="AQ9" s="37" t="n">
         <f aca="false">IF(AND($O9=1,$T9&gt;0),Pipeline!$T9/$T9,0)</f>
-        <v>0.0285204991087344</v>
+        <v>0.0313725490196078</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6897,7 +6897,7 @@
       </c>
       <c r="S12" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q12+$R12,MaxSupportPct*Pipeline!$N12-Pipeline!$Q12,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>399000</v>
+        <v>382500</v>
       </c>
       <c r="T12" s="28" t="n">
         <f aca="false">IF($O12=1,IF(Pipeline!$V12&gt;0,MIN(Pipeline!$V12,$S12),$S12),0)</f>
@@ -7245,11 +7245,11 @@
       </c>
       <c r="S14" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q14+$R14,MaxSupportPct*Pipeline!$N14-Pipeline!$Q14,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T14" s="28" t="n">
         <f aca="false">IF($O14=1,IF(Pipeline!$V14&gt;0,MIN(Pipeline!$V14,$S14),$S14),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U14" s="29" t="n">
         <f aca="false">IFERROR($Q14/($Q14+$R14),1)</f>
@@ -7257,15 +7257,15 @@
       </c>
       <c r="V14" s="28" t="n">
         <f aca="false">IFERROR($T14/$C14,0)</f>
-        <v>480.308219178082</v>
+        <v>436.643835616438</v>
       </c>
       <c r="W14" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O14+Pipeline!$P14)/$T14,0)</f>
-        <v>1.42602495543672</v>
+        <v>1.56862745098039</v>
       </c>
       <c r="X14" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T14/$T14*1000,0)</f>
-        <v>15.4486036838978</v>
+        <v>16.9934640522876</v>
       </c>
       <c r="Y14" s="30" t="str">
         <f aca="false">IF($O14=0,"",IF(NOT(ISNUMBER(Pipeline!$U14)),"No viability-gap data",IF(Pipeline!$U14&lt;=0,"No viability-gap data",IF($T14&lt;=Pipeline!$U14*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="AK14" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,8,Allocation!$I$7:$I$31)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="AL14" s="29" t="n">
         <f aca="false">IFERROR($AK14/$T14,0)</f>
@@ -7329,11 +7329,11 @@
       </c>
       <c r="AN14" s="37" t="n">
         <f aca="false">IF(AND($O14=1,$V14&gt;0),1/$V14,0)</f>
-        <v>0.00208199643493761</v>
+        <v>0.00229019607843137</v>
       </c>
       <c r="AO14" s="38" t="n">
         <f aca="false">IF($O14=1,$W14,0)</f>
-        <v>1.42602495543672</v>
+        <v>1.56862745098039</v>
       </c>
       <c r="AP14" s="39" t="n">
         <f aca="false">IF($O14=1,$F14,0)</f>
@@ -7341,7 +7341,7 @@
       </c>
       <c r="AQ14" s="37" t="n">
         <f aca="false">IF(AND($O14=1,$T14&gt;0),Pipeline!$T14/$T14,0)</f>
-        <v>0.0154486036838978</v>
+        <v>0.0169934640522876</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7419,11 +7419,11 @@
       </c>
       <c r="S15" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q15+$R15,MaxSupportPct*Pipeline!$N15-Pipeline!$Q15,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>403250</v>
+        <v>382500</v>
       </c>
       <c r="T15" s="28" t="n">
         <f aca="false">IF($O15=1,IF(Pipeline!$V15&gt;0,MIN(Pipeline!$V15,$S15),$S15),0)</f>
-        <v>403250</v>
+        <v>382500</v>
       </c>
       <c r="U15" s="29" t="n">
         <f aca="false">IFERROR($Q15/($Q15+$R15),1)</f>
@@ -7431,15 +7431,15 @@
       </c>
       <c r="V15" s="28" t="n">
         <f aca="false">IFERROR($T15/$C15,0)</f>
-        <v>439.749182115594</v>
+        <v>417.121046892039</v>
       </c>
       <c r="W15" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O15+Pipeline!$P15)/$T15,0)</f>
-        <v>0.867947923124613</v>
+        <v>0.915032679738562</v>
       </c>
       <c r="X15" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T15/$T15*1000,0)</f>
-        <v>12.3992560446373</v>
+        <v>13.0718954248366</v>
       </c>
       <c r="Y15" s="30" t="str">
         <f aca="false">IF($O15=0,"",IF(NOT(ISNUMBER(Pipeline!$U15)),"No viability-gap data",IF(Pipeline!$U15&lt;=0,"No viability-gap data",IF($T15&lt;=Pipeline!$U15*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -7447,11 +7447,11 @@
       </c>
       <c r="Z15" s="33" t="n">
         <f aca="false">IF($O15=1,IFERROR($AN15/MAX($AN$7:$AN$31)*100,0),0)</f>
-        <v>55.8223694442978</v>
+        <v>53.5005834305718</v>
       </c>
       <c r="AA15" s="33" t="n">
         <f aca="false">IF($O15=1,IFERROR($AO15/MAX($AO$7:$AO$31)*100,0),0)</f>
-        <v>36.5189088654681</v>
+        <v>35</v>
       </c>
       <c r="AB15" s="33" t="n">
         <f aca="false">IF($O15=1,IFERROR($AP15/MAX($AP$7:$AP$31)*100,0),0)</f>
@@ -7459,7 +7459,7 @@
       </c>
       <c r="AC15" s="33" t="n">
         <f aca="false">IF($O15=1,IFERROR($AQ15/MAX($AQ$7:$AQ$31)*100,0),0)</f>
-        <v>43.4748915065096</v>
+        <v>41.6666666666667</v>
       </c>
       <c r="AD15" s="33" t="n">
         <f aca="false">IF($O15=1,Pipeline!$F15/5*100,0)</f>
@@ -7479,35 +7479,35 @@
       </c>
       <c r="AH15" s="34" t="n">
         <f aca="false">$Z15*W_Cost+$AA15*W_Lev+$AB15*W_PU+$AC15*W_CO2+$AD15*W_Ready+$AE15*W_Track+$AF15*W_Risk+$AG15*W_Add</f>
-        <v>53.9455852352206</v>
+        <v>52.9564799179846</v>
       </c>
       <c r="AI15" s="35" t="n">
         <f aca="false">IF($O15=1,$AH15+(26-$A15)/1000000,-1)</f>
-        <v>53.9456022352206</v>
+        <v>52.9564969179846</v>
       </c>
       <c r="AJ15" s="21" t="n">
         <f aca="false">IF($O15=1,COUNTIF($AI$7:$AI$31,"&gt;"&amp;$AI15)+1,"")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AK15" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,9,Allocation!$I$7:$I$31)</f>
-        <v>241000</v>
+        <v>382500</v>
       </c>
       <c r="AL15" s="29" t="n">
         <f aca="false">IFERROR($AK15/$T15,0)</f>
-        <v>0.597644141351519</v>
+        <v>1</v>
       </c>
       <c r="AM15" s="30" t="str">
         <f aca="false">IF($O15=0,"",IF($AL15&gt;=0.999,"Funded",IF($AK15&gt;0,"Partially funded","Not funded")))</f>
-        <v>Partially funded</v>
+        <v>Funded</v>
       </c>
       <c r="AN15" s="37" t="n">
         <f aca="false">IF(AND($O15=1,$V15&gt;0),1/$V15,0)</f>
-        <v>0.00227402355858649</v>
+        <v>0.00239738562091503</v>
       </c>
       <c r="AO15" s="38" t="n">
         <f aca="false">IF($O15=1,$W15,0)</f>
-        <v>0.867947923124613</v>
+        <v>0.915032679738562</v>
       </c>
       <c r="AP15" s="39" t="n">
         <f aca="false">IF($O15=1,$F15,0)</f>
@@ -7515,7 +7515,7 @@
       </c>
       <c r="AQ15" s="37" t="n">
         <f aca="false">IF(AND($O15=1,$T15&gt;0),Pipeline!$T15/$T15,0)</f>
-        <v>0.0123992560446373</v>
+        <v>0.0130718954248366</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7767,11 +7767,11 @@
       </c>
       <c r="S17" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q17+$R17,MaxSupportPct*Pipeline!$N17-Pipeline!$Q17,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T17" s="28" t="n">
         <f aca="false">IF($O17=1,IF(Pipeline!$V17&gt;0,MIN(Pipeline!$V17,$S17),$S17),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U17" s="29" t="n">
         <f aca="false">IFERROR($Q17/($Q17+$R17),1)</f>
@@ -7779,15 +7779,15 @@
       </c>
       <c r="V17" s="28" t="n">
         <f aca="false">IFERROR($T17/$C17,0)</f>
-        <v>288.184931506849</v>
+        <v>261.986301369863</v>
       </c>
       <c r="W17" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O17+Pipeline!$P17)/$T17,0)</f>
-        <v>1.90136660724896</v>
+        <v>2.09150326797386</v>
       </c>
       <c r="X17" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T17/$T17*1000,0)</f>
-        <v>19.0136660724896</v>
+        <v>20.9150326797386</v>
       </c>
       <c r="Y17" s="30" t="str">
         <f aca="false">IF($O17=0,"",IF(NOT(ISNUMBER(Pipeline!$U17)),"No viability-gap data",IF(Pipeline!$U17&lt;=0,"No viability-gap data",IF($T17&lt;=Pipeline!$U17*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="AK17" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,11,Allocation!$I$7:$I$31)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="AL17" s="29" t="n">
         <f aca="false">IFERROR($AK17/$T17,0)</f>
@@ -7851,11 +7851,11 @@
       </c>
       <c r="AN17" s="37" t="n">
         <f aca="false">IF(AND($O17=1,$V17&gt;0),1/$V17,0)</f>
-        <v>0.00346999405822935</v>
+        <v>0.00381699346405229</v>
       </c>
       <c r="AO17" s="38" t="n">
         <f aca="false">IF($O17=1,$W17,0)</f>
-        <v>1.90136660724896</v>
+        <v>2.09150326797386</v>
       </c>
       <c r="AP17" s="39" t="n">
         <f aca="false">IF($O17=1,$F17,0)</f>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="AQ17" s="37" t="n">
         <f aca="false">IF(AND($O17=1,$T17&gt;0),Pipeline!$T17/$T17,0)</f>
-        <v>0.0190136660724896</v>
+        <v>0.0209150326797386</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7941,11 +7941,11 @@
       </c>
       <c r="S18" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q18+$R18,MaxSupportPct*Pipeline!$N18-Pipeline!$Q18,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T18" s="28" t="n">
         <f aca="false">IF($O18=1,IF(Pipeline!$V18&gt;0,MIN(Pipeline!$V18,$S18),$S18),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U18" s="29" t="n">
         <f aca="false">IFERROR($Q18/($Q18+$R18),1)</f>
@@ -7953,15 +7953,15 @@
       </c>
       <c r="V18" s="28" t="n">
         <f aca="false">IFERROR($T18/$C18,0)</f>
-        <v>324.152542372881</v>
+        <v>294.684129429892</v>
       </c>
       <c r="W18" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O18+Pipeline!$P18)/$T18,0)</f>
-        <v>1.66369578134284</v>
+        <v>1.83006535947712</v>
       </c>
       <c r="X18" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T18/$T18*1000,0)</f>
-        <v>17.825311942959</v>
+        <v>19.6078431372549</v>
       </c>
       <c r="Y18" s="30" t="str">
         <f aca="false">IF($O18=0,"",IF(NOT(ISNUMBER(Pipeline!$U18)),"No viability-gap data",IF(Pipeline!$U18&lt;=0,"No viability-gap data",IF($T18&lt;=Pipeline!$U18*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -8013,7 +8013,7 @@
       </c>
       <c r="AK18" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,12,Allocation!$I$7:$I$31)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="AL18" s="29" t="n">
         <f aca="false">IFERROR($AK18/$T18,0)</f>
@@ -8025,11 +8025,11 @@
       </c>
       <c r="AN18" s="37" t="n">
         <f aca="false">IF(AND($O18=1,$V18&gt;0),1/$V18,0)</f>
-        <v>0.00308496732026144</v>
+        <v>0.00339346405228758</v>
       </c>
       <c r="AO18" s="38" t="n">
         <f aca="false">IF($O18=1,$W18,0)</f>
-        <v>1.66369578134284</v>
+        <v>1.83006535947712</v>
       </c>
       <c r="AP18" s="39" t="n">
         <f aca="false">IF($O18=1,$F18,0)</f>
@@ -8037,7 +8037,7 @@
       </c>
       <c r="AQ18" s="37" t="n">
         <f aca="false">IF(AND($O18=1,$T18&gt;0),Pipeline!$T18/$T18,0)</f>
-        <v>0.017825311942959</v>
+        <v>0.0196078431372549</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8289,11 +8289,11 @@
       </c>
       <c r="S20" s="28" t="n">
         <f aca="false">MAX(0,MIN($Q20+$R20,MaxSupportPct*Pipeline!$N20-Pipeline!$Q20,MaxPerProject,MaxProjShare*Envelope))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="T20" s="28" t="n">
         <f aca="false">IF($O20=1,IF(Pipeline!$V20&gt;0,MIN(Pipeline!$V20,$S20),$S20),0)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="U20" s="29" t="n">
         <f aca="false">IFERROR($Q20/($Q20+$R20),1)</f>
@@ -8301,15 +8301,15 @@
       </c>
       <c r="V20" s="28" t="n">
         <f aca="false">IFERROR($T20/$C20,0)</f>
-        <v>414.940828402367</v>
+        <v>377.218934911243</v>
       </c>
       <c r="W20" s="31" t="n">
         <f aca="false">IFERROR((Pipeline!$O20+Pipeline!$P20)/$T20,0)</f>
-        <v>1.30718954248366</v>
+        <v>1.43790849673203</v>
       </c>
       <c r="X20" s="32" t="n">
         <f aca="false">IFERROR(Pipeline!$T20/$T20*1000,0)</f>
-        <v>16.1616161616162</v>
+        <v>17.7777777777778</v>
       </c>
       <c r="Y20" s="30" t="str">
         <f aca="false">IF($O20=0,"",IF(NOT(ISNUMBER(Pipeline!$U20)),"No viability-gap data",IF(Pipeline!$U20&lt;=0,"No viability-gap data",IF($T20&lt;=Pipeline!$U20*(1+VGFTol),"Within viability gap","Above viability gap"))))</f>
@@ -8361,7 +8361,7 @@
       </c>
       <c r="AK20" s="36" t="n">
         <f aca="false">SUMIF(Allocation!$B$7:$B$31,14,Allocation!$I$7:$I$31)</f>
-        <v>140250</v>
+        <v>127500</v>
       </c>
       <c r="AL20" s="29" t="n">
         <f aca="false">IFERROR($AK20/$T20,0)</f>
@@ -8373,11 +8373,11 @@
       </c>
       <c r="AN20" s="37" t="n">
         <f aca="false">IF(AND($O20=1,$V20&gt;0),1/$V20,0)</f>
-        <v>0.00240998217468806</v>
+        <v>0.00265098039215686</v>
       </c>
       <c r="AO20" s="38" t="n">
         <f aca="false">IF($O20=1,$W20,0)</f>
-        <v>1.30718954248366</v>
+        <v>1.43790849673203</v>
       </c>
       <c r="AP20" s="39" t="n">
         <f aca="false">IF($O20=1,$F20,0)</f>
@@ -8385,7 +8385,7 @@
       </c>
       <c r="AQ20" s="37" t="n">
         <f aca="false">IF(AND($O20=1,$T20&gt;0),Pipeline!$T20/$T20,0)</f>
-        <v>0.0161616161616162</v>
+        <v>0.0177777777777778</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10362,7 +10362,7 @@
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="40" t="str">
         <f aca="false">"Envelope: "&amp;Currency&amp;" "&amp;FIXED(Envelope,0)&amp;"  |  Partial funding: "&amp;IF(AllowPartial=1,"allowed","not allowed")&amp;"  |  Max per country: "&amp;FIXED((MaxCountryShare)*100,0)&amp;"%"&amp;" of envelope"</f>
-        <v>Envelope: USD 2,805,000  |  Partial funding: allowed  |  Max per country: 50% of envelope</v>
+        <v>Envelope: USD 2,550,000  |  Partial funding: allowed  |  Max per country: 50% of envelope</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10428,19 +10428,19 @@
       </c>
       <c r="F7" s="36" t="n">
         <f aca="false">IF(B7="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B7))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G7" s="28" t="n">
         <f aca="false">IF(B7="","",Envelope)</f>
-        <v>2805000</v>
+        <v>2550000</v>
       </c>
       <c r="H7" s="28" t="n">
         <f aca="false">IF(B7="","",MaxCountryShare*Envelope)</f>
-        <v>1402500</v>
+        <v>1275000</v>
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">IF(B7="",0,IF(AllowPartial=1,MAX(0,MIN(F7,G7,H7)),IF(F7&lt;=MIN(G7,H7),F7,0)))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="J7" s="30" t="str">
         <f aca="false">IF(B7="","",IF(I7&gt;=F7-0.5,"Funded",IF(I7&gt;0,"Partially funded","Not funded")))</f>
@@ -10474,19 +10474,19 @@
       </c>
       <c r="F8" s="36" t="n">
         <f aca="false">IF(B8="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B8))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">IF(B8="","",Envelope-SUM($I$7:I7))</f>
-        <v>2384250</v>
+        <v>2167500</v>
       </c>
       <c r="H8" s="28" t="n">
         <f aca="false">IF(B8="","",MaxCountryShare*Envelope-SUMIF($D$7:D7,D8,$I$7:I7))</f>
-        <v>981750</v>
+        <v>892500</v>
       </c>
       <c r="I8" s="16" t="n">
         <f aca="false">IF(B8="",0,IF(AllowPartial=1,MAX(0,MIN(F8,G8,H8)),IF(F8&lt;=MIN(G8,H8),F8,0)))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="J8" s="30" t="str">
         <f aca="false">IF(B8="","",IF(I8&gt;=F8-0.5,"Funded",IF(I8&gt;0,"Partially funded","Not funded")))</f>
@@ -10520,19 +10520,19 @@
       </c>
       <c r="F9" s="36" t="n">
         <f aca="false">IF(B9="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B9))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">IF(B9="","",Envelope-SUM($I$7:I8))</f>
-        <v>1963500</v>
+        <v>1785000</v>
       </c>
       <c r="H9" s="28" t="n">
         <f aca="false">IF(B9="","",MaxCountryShare*Envelope-SUMIF($D$7:D8,D9,$I$7:I8))</f>
-        <v>1402500</v>
+        <v>1275000</v>
       </c>
       <c r="I9" s="16" t="n">
         <f aca="false">IF(B9="",0,IF(AllowPartial=1,MAX(0,MIN(F9,G9,H9)),IF(F9&lt;=MIN(G9,H9),F9,0)))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="J9" s="30" t="str">
         <f aca="false">IF(B9="","",IF(I9&gt;=F9-0.5,"Funded",IF(I9&gt;0,"Partially funded","Not funded")))</f>
@@ -10566,19 +10566,19 @@
       </c>
       <c r="F10" s="36" t="n">
         <f aca="false">IF(B10="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B10))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G10" s="28" t="n">
         <f aca="false">IF(B10="","",Envelope-SUM($I$7:I9))</f>
-        <v>1542750</v>
+        <v>1402500</v>
       </c>
       <c r="H10" s="28" t="n">
         <f aca="false">IF(B10="","",MaxCountryShare*Envelope-SUMIF($D$7:D9,D10,$I$7:I9))</f>
-        <v>561000</v>
+        <v>510000</v>
       </c>
       <c r="I10" s="16" t="n">
         <f aca="false">IF(B10="",0,IF(AllowPartial=1,MAX(0,MIN(F10,G10,H10)),IF(F10&lt;=MIN(G10,H10),F10,0)))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="J10" s="30" t="str">
         <f aca="false">IF(B10="","",IF(I10&gt;=F10-0.5,"Funded",IF(I10&gt;0,"Partially funded","Not funded")))</f>
@@ -10612,19 +10612,19 @@
       </c>
       <c r="F11" s="36" t="n">
         <f aca="false">IF(B11="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B11))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G11" s="28" t="n">
         <f aca="false">IF(B11="","",Envelope-SUM($I$7:I10))</f>
-        <v>1122000</v>
+        <v>1020000</v>
       </c>
       <c r="H11" s="28" t="n">
         <f aca="false">IF(B11="","",MaxCountryShare*Envelope-SUMIF($D$7:D10,D11,$I$7:I10))</f>
-        <v>1402500</v>
+        <v>1275000</v>
       </c>
       <c r="I11" s="16" t="n">
         <f aca="false">IF(B11="",0,IF(AllowPartial=1,MAX(0,MIN(F11,G11,H11)),IF(F11&lt;=MIN(G11,H11),F11,0)))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="J11" s="30" t="str">
         <f aca="false">IF(B11="","",IF(I11&gt;=F11-0.5,"Funded",IF(I11&gt;0,"Partially funded","Not funded")))</f>
@@ -10658,19 +10658,19 @@
       </c>
       <c r="F12" s="36" t="n">
         <f aca="false">IF(B12="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B12))</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G12" s="28" t="n">
         <f aca="false">IF(B12="","",Envelope-SUM($I$7:I11))</f>
-        <v>701250</v>
+        <v>637500</v>
       </c>
       <c r="H12" s="28" t="n">
         <f aca="false">IF(B12="","",MaxCountryShare*Envelope-SUMIF($D$7:D11,D12,$I$7:I11))</f>
-        <v>140250</v>
+        <v>127500</v>
       </c>
       <c r="I12" s="16" t="n">
         <f aca="false">IF(B12="",0,IF(AllowPartial=1,MAX(0,MIN(F12,G12,H12)),IF(F12&lt;=MIN(G12,H12),F12,0)))</f>
-        <v>140250</v>
+        <v>127500</v>
       </c>
       <c r="J12" s="30" t="str">
         <f aca="false">IF(B12="","",IF(I12&gt;=F12-0.5,"Funded",IF(I12&gt;0,"Partially funded","Not funded")))</f>
@@ -10688,35 +10688,35 @@
       </c>
       <c r="B13" s="25" t="n">
         <f aca="false">IFERROR(MATCH(7,'Eligibility &amp; Scoring'!$AJ$7:$AJ$31,0),"")</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C13" s="26" t="str">
         <f aca="false">IF(B13="","",INDEX('Eligibility &amp; Scoring'!$B$7:$B$31,B13))</f>
-        <v>Project B - River towns</v>
+        <v>Project I - Fishing communities</v>
       </c>
       <c r="D13" s="26" t="str">
         <f aca="false">IF(B13="","",INDEX(Pipeline!$C$7:$C$31,B13))</f>
-        <v>Country A</v>
+        <v>Country D</v>
       </c>
       <c r="E13" s="41" t="n">
         <f aca="false">IF(B13="",0,INDEX('Eligibility &amp; Scoring'!$AH$7:$AH$31,B13))</f>
-        <v>54.2270489630815</v>
+        <v>52.9564799179846</v>
       </c>
       <c r="F13" s="36" t="n">
         <f aca="false">IF(B13="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B13))</f>
-        <v>320000</v>
+        <v>382500</v>
       </c>
       <c r="G13" s="28" t="n">
         <f aca="false">IF(B13="","",Envelope-SUM($I$7:I12))</f>
-        <v>561000</v>
+        <v>510000</v>
       </c>
       <c r="H13" s="28" t="n">
         <f aca="false">IF(B13="","",MaxCountryShare*Envelope-SUMIF($D$7:D12,D13,$I$7:I12))</f>
-        <v>981750</v>
+        <v>892500</v>
       </c>
       <c r="I13" s="16" t="n">
         <f aca="false">IF(B13="",0,IF(AllowPartial=1,MAX(0,MIN(F13,G13,H13)),IF(F13&lt;=MIN(G13,H13),F13,0)))</f>
-        <v>320000</v>
+        <v>382500</v>
       </c>
       <c r="J13" s="30" t="str">
         <f aca="false">IF(B13="","",IF(I13&gt;=F13-0.5,"Funded",IF(I13&gt;0,"Partially funded","Not funded")))</f>
@@ -10734,35 +10734,35 @@
       </c>
       <c r="B14" s="25" t="n">
         <f aca="false">IFERROR(MATCH(8,'Eligibility &amp; Scoring'!$AJ$7:$AJ$31,0),"")</f>
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C14" s="26" t="str">
         <f aca="false">IF(B14="","",INDEX('Eligibility &amp; Scoring'!$B$7:$B$31,B14))</f>
-        <v>Project I - Fishing communities</v>
+        <v>Project B - River towns</v>
       </c>
       <c r="D14" s="26" t="str">
         <f aca="false">IF(B14="","",INDEX(Pipeline!$C$7:$C$31,B14))</f>
-        <v>Country D</v>
+        <v>Country A</v>
       </c>
       <c r="E14" s="41" t="n">
         <f aca="false">IF(B14="",0,INDEX('Eligibility &amp; Scoring'!$AH$7:$AH$31,B14))</f>
-        <v>53.9455852352206</v>
+        <v>51.9378232848435</v>
       </c>
       <c r="F14" s="36" t="n">
         <f aca="false">IF(B14="",0,INDEX('Eligibility &amp; Scoring'!$T$7:$T$31,B14))</f>
-        <v>403250</v>
+        <v>320000</v>
       </c>
       <c r="G14" s="28" t="n">
         <f aca="false">IF(B14="","",Envelope-SUM($I$7:I13))</f>
-        <v>241000</v>
+        <v>127500</v>
       </c>
       <c r="H14" s="28" t="n">
         <f aca="false">IF(B14="","",MaxCountryShare*Envelope-SUMIF($D$7:D13,D14,$I$7:I13))</f>
-        <v>981750</v>
+        <v>892500</v>
       </c>
       <c r="I14" s="16" t="n">
         <f aca="false">IF(B14="",0,IF(AllowPartial=1,MAX(0,MIN(F14,G14,H14)),IF(F14&lt;=MIN(G14,H14),F14,0)))</f>
-        <v>241000</v>
+        <v>127500</v>
       </c>
       <c r="J14" s="30" t="str">
         <f aca="false">IF(B14="","",IF(I14&gt;=F14-0.5,"Funded",IF(I14&gt;0,"Partially funded","Not funded")))</f>
@@ -11561,11 +11561,11 @@
       </c>
       <c r="F32" s="43" t="n">
         <f aca="false">SUM(F7:F31)</f>
-        <v>3247750</v>
+        <v>2997500</v>
       </c>
       <c r="I32" s="43" t="n">
         <f aca="false">SUM(I7:I31)</f>
-        <v>2805000</v>
+        <v>2550000</v>
       </c>
     </row>
   </sheetData>
@@ -11709,11 +11709,11 @@
       </c>
       <c r="C6" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7*'Eligibility &amp; Scoring'!$U7</f>
-        <v>121856.557377049</v>
+        <v>110778.68852459</v>
       </c>
       <c r="D6" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7-C6</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
       <c r="E6" s="29" t="n">
         <f aca="false">IF(C6+D6=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H7),1))</f>
@@ -11721,23 +11721,23 @@
       </c>
       <c r="F6" s="28" t="n">
         <f aca="false">C6*E6</f>
-        <v>115763.729508197</v>
+        <v>105239.754098361</v>
       </c>
       <c r="G6" s="47" t="n">
         <f aca="false">$C6*$E6*(TrancheA*IF(1-VerifLag=Pipeline!$I7,RampV1,IF(1-VerifLag=Pipeline!$I7+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I7+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I7,RampV1,IF(1-VerifLag-1=Pipeline!$I7+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I7+2,1-RampV2,0))))</f>
-        <v>48620.7663934426</v>
+        <v>44200.6967213115</v>
       </c>
       <c r="H6" s="47" t="n">
         <f aca="false">$C6*$E6*(TrancheA*IF(2-VerifLag=Pipeline!$I7,RampV1,IF(2-VerifLag=Pipeline!$I7+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I7+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I7,RampV1,IF(2-VerifLag-1=Pipeline!$I7+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I7+2,1-RampV2,0))))</f>
-        <v>45147.8545081967</v>
+        <v>41043.5040983607</v>
       </c>
       <c r="I6" s="47" t="n">
         <f aca="false">$C6*$E6*(TrancheA*IF(3-VerifLag=Pipeline!$I7,RampV1,IF(3-VerifLag=Pipeline!$I7+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I7+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I7,RampV1,IF(3-VerifLag-1=Pipeline!$I7+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I7+2,1-RampV2,0))))</f>
-        <v>18522.1967213115</v>
+        <v>16838.3606557377</v>
       </c>
       <c r="J6" s="47" t="n">
         <f aca="false">$C6*$E6*(TrancheA*IF(4-VerifLag=Pipeline!$I7,RampV1,IF(4-VerifLag=Pipeline!$I7+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I7+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I7,RampV1,IF(4-VerifLag-1=Pipeline!$I7+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I7+2,1-RampV2,0))))</f>
-        <v>3472.9118852459</v>
+        <v>3157.19262295082</v>
       </c>
       <c r="K6" s="47" t="n">
         <f aca="false">$C6*$E6*(TrancheA*IF(5-VerifLag=Pipeline!$I7,RampV1,IF(5-VerifLag=Pipeline!$I7+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I7+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I7,RampV1,IF(5-VerifLag-1=Pipeline!$I7+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I7+2,1-RampV2,0))))</f>
@@ -11765,7 +11765,7 @@
       </c>
       <c r="Q6" s="48" t="n">
         <f aca="false">SUM(G6:P6)</f>
-        <v>115763.729508197</v>
+        <v>105239.754098361</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11778,11 +11778,11 @@
       </c>
       <c r="C7" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8*'Eligibility &amp; Scoring'!$U8</f>
-        <v>82500</v>
+        <v>32871.09375</v>
       </c>
       <c r="D7" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8-C7</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
       <c r="E7" s="29" t="n">
         <f aca="false">IF(C7+D7=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H8),1))</f>
@@ -11790,7 +11790,7 @@
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">C7*E7</f>
-        <v>74250</v>
+        <v>29583.984375</v>
       </c>
       <c r="G7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(1-VerifLag=Pipeline!$I8,RampV1,IF(1-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I8,RampV1,IF(1-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
@@ -11798,19 +11798,19 @@
       </c>
       <c r="H7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(2-VerifLag=Pipeline!$I8,RampV1,IF(2-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I8,RampV1,IF(2-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
-        <v>31185</v>
+        <v>12425.2734375</v>
       </c>
       <c r="I7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(3-VerifLag=Pipeline!$I8,RampV1,IF(3-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I8,RampV1,IF(3-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
-        <v>28957.5</v>
+        <v>11537.75390625</v>
       </c>
       <c r="J7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(4-VerifLag=Pipeline!$I8,RampV1,IF(4-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I8,RampV1,IF(4-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
-        <v>11880</v>
+        <v>4733.4375</v>
       </c>
       <c r="K7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(5-VerifLag=Pipeline!$I8,RampV1,IF(5-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I8,RampV1,IF(5-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
-        <v>2227.5</v>
+        <v>887.51953125</v>
       </c>
       <c r="L7" s="47" t="n">
         <f aca="false">$C7*$E7*(TrancheA*IF(6-VerifLag=Pipeline!$I8,RampV1,IF(6-VerifLag=Pipeline!$I8+1,RampV2-RampV1,IF(6-VerifLag=Pipeline!$I8+2,1-RampV2,0)))+(1-TrancheA)*IF(6-VerifLag-1=Pipeline!$I8,RampV1,IF(6-VerifLag-1=Pipeline!$I8+1,RampV2-RampV1,IF(6-VerifLag-1=Pipeline!$I8+2,1-RampV2,0))))</f>
@@ -11834,7 +11834,7 @@
       </c>
       <c r="Q7" s="48" t="n">
         <f aca="false">SUM(G7:P7)</f>
-        <v>74250</v>
+        <v>29583.984375</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11847,11 +11847,11 @@
       </c>
       <c r="C8" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9*'Eligibility &amp; Scoring'!$U9</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
       <c r="D8" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9-C8</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
       <c r="E8" s="29" t="n">
         <f aca="false">IF(C8+D8=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H9),1))</f>
@@ -11859,23 +11859,23 @@
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">C8*E8</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
       <c r="G8" s="47" t="n">
         <f aca="false">$C8*$E8*(TrancheA*IF(1-VerifLag=Pipeline!$I9,RampV1,IF(1-VerifLag=Pipeline!$I9+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I9+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I9,RampV1,IF(1-VerifLag-1=Pipeline!$I9+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I9+2,1-RampV2,0))))</f>
-        <v>53224.4339622642</v>
+        <v>48385.8490566038</v>
       </c>
       <c r="H8" s="47" t="n">
         <f aca="false">$C8*$E8*(TrancheA*IF(2-VerifLag=Pipeline!$I9,RampV1,IF(2-VerifLag=Pipeline!$I9+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I9+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I9,RampV1,IF(2-VerifLag-1=Pipeline!$I9+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I9+2,1-RampV2,0))))</f>
-        <v>49422.6886792453</v>
+        <v>44929.7169811321</v>
       </c>
       <c r="I8" s="47" t="n">
         <f aca="false">$C8*$E8*(TrancheA*IF(3-VerifLag=Pipeline!$I9,RampV1,IF(3-VerifLag=Pipeline!$I9+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I9+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I9,RampV1,IF(3-VerifLag-1=Pipeline!$I9+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I9+2,1-RampV2,0))))</f>
-        <v>20275.9748427673</v>
+        <v>18432.7044025157</v>
       </c>
       <c r="J8" s="47" t="n">
         <f aca="false">$C8*$E8*(TrancheA*IF(4-VerifLag=Pipeline!$I9,RampV1,IF(4-VerifLag=Pipeline!$I9+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I9+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I9,RampV1,IF(4-VerifLag-1=Pipeline!$I9+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I9+2,1-RampV2,0))))</f>
-        <v>3801.74528301887</v>
+        <v>3456.1320754717</v>
       </c>
       <c r="K8" s="47" t="n">
         <f aca="false">$C8*$E8*(TrancheA*IF(5-VerifLag=Pipeline!$I9,RampV1,IF(5-VerifLag=Pipeline!$I9+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I9+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I9,RampV1,IF(5-VerifLag-1=Pipeline!$I9+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I9+2,1-RampV2,0))))</f>
@@ -11903,7 +11903,7 @@
       </c>
       <c r="Q8" s="48" t="n">
         <f aca="false">SUM(G8:P8)</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12192,11 +12192,11 @@
       </c>
       <c r="C13" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14*'Eligibility &amp; Scoring'!$U14</f>
-        <v>123400.176678445</v>
+        <v>112181.978798587</v>
       </c>
       <c r="D13" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14-C13</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
       <c r="E13" s="29" t="n">
         <f aca="false">IF(C13+D13=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H14),1))</f>
@@ -12204,7 +12204,7 @@
       </c>
       <c r="F13" s="28" t="n">
         <f aca="false">C13*E13</f>
-        <v>117230.167844523</v>
+        <v>106572.879858657</v>
       </c>
       <c r="G13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(1-VerifLag=Pipeline!$I14,RampV1,IF(1-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I14,RampV1,IF(1-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
@@ -12212,19 +12212,19 @@
       </c>
       <c r="H13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(2-VerifLag=Pipeline!$I14,RampV1,IF(2-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I14,RampV1,IF(2-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
-        <v>49236.6704946996</v>
+        <v>44760.609540636</v>
       </c>
       <c r="I13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(3-VerifLag=Pipeline!$I14,RampV1,IF(3-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I14,RampV1,IF(3-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
-        <v>45719.765459364</v>
+        <v>41563.4231448763</v>
       </c>
       <c r="J13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(4-VerifLag=Pipeline!$I14,RampV1,IF(4-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I14,RampV1,IF(4-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
-        <v>18756.8268551237</v>
+        <v>17051.6607773852</v>
       </c>
       <c r="K13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(5-VerifLag=Pipeline!$I14,RampV1,IF(5-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I14,RampV1,IF(5-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
-        <v>3516.90503533569</v>
+        <v>3197.18639575972</v>
       </c>
       <c r="L13" s="47" t="n">
         <f aca="false">$C13*$E13*(TrancheA*IF(6-VerifLag=Pipeline!$I14,RampV1,IF(6-VerifLag=Pipeline!$I14+1,RampV2-RampV1,IF(6-VerifLag=Pipeline!$I14+2,1-RampV2,0)))+(1-TrancheA)*IF(6-VerifLag-1=Pipeline!$I14,RampV1,IF(6-VerifLag-1=Pipeline!$I14+1,RampV2-RampV1,IF(6-VerifLag-1=Pipeline!$I14+2,1-RampV2,0))))</f>
@@ -12248,7 +12248,7 @@
       </c>
       <c r="Q13" s="48" t="n">
         <f aca="false">SUM(G13:P13)</f>
-        <v>117230.167844523</v>
+        <v>106572.879858657</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12261,11 +12261,11 @@
       </c>
       <c r="C14" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15*'Eligibility &amp; Scoring'!$U15</f>
-        <v>69177.3093614383</v>
+        <v>109793.862368258</v>
       </c>
       <c r="D14" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15-C14</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
       <c r="E14" s="29" t="n">
         <f aca="false">IF(C14+D14=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H15),1))</f>
@@ -12273,7 +12273,7 @@
       </c>
       <c r="F14" s="28" t="n">
         <f aca="false">C14*E14</f>
-        <v>62259.5784252945</v>
+        <v>98814.4761314321</v>
       </c>
       <c r="G14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(1-VerifLag=Pipeline!$I15,RampV1,IF(1-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I15,RampV1,IF(1-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
@@ -12281,19 +12281,19 @@
       </c>
       <c r="H14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(2-VerifLag=Pipeline!$I15,RampV1,IF(2-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I15,RampV1,IF(2-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
-        <v>26149.0229386237</v>
+        <v>41502.0799752015</v>
       </c>
       <c r="I14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(3-VerifLag=Pipeline!$I15,RampV1,IF(3-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I15,RampV1,IF(3-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
-        <v>24281.2355858648</v>
+        <v>38537.6456912585</v>
       </c>
       <c r="J14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(4-VerifLag=Pipeline!$I15,RampV1,IF(4-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I15,RampV1,IF(4-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
-        <v>9961.53254804712</v>
+        <v>15810.3161810291</v>
       </c>
       <c r="K14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(5-VerifLag=Pipeline!$I15,RampV1,IF(5-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I15,RampV1,IF(5-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
-        <v>1867.78735275883</v>
+        <v>2964.43428394296</v>
       </c>
       <c r="L14" s="47" t="n">
         <f aca="false">$C14*$E14*(TrancheA*IF(6-VerifLag=Pipeline!$I15,RampV1,IF(6-VerifLag=Pipeline!$I15+1,RampV2-RampV1,IF(6-VerifLag=Pipeline!$I15+2,1-RampV2,0)))+(1-TrancheA)*IF(6-VerifLag-1=Pipeline!$I15,RampV1,IF(6-VerifLag-1=Pipeline!$I15+1,RampV2-RampV1,IF(6-VerifLag-1=Pipeline!$I15+2,1-RampV2,0))))</f>
@@ -12317,7 +12317,7 @@
       </c>
       <c r="Q14" s="48" t="n">
         <f aca="false">SUM(G14:P14)</f>
-        <v>62259.5784252945</v>
+        <v>98814.4761314321</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12399,11 +12399,11 @@
       </c>
       <c r="C16" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17*'Eligibility &amp; Scoring'!$U17</f>
-        <v>137225.741239892</v>
+        <v>124750.673854447</v>
       </c>
       <c r="D16" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17-C16</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
       <c r="E16" s="29" t="n">
         <f aca="false">IF(C16+D16=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H17),1))</f>
@@ -12411,23 +12411,23 @@
       </c>
       <c r="F16" s="28" t="n">
         <f aca="false">C16*E16</f>
-        <v>130364.454177898</v>
+        <v>118513.140161725</v>
       </c>
       <c r="G16" s="47" t="n">
         <f aca="false">$C16*$E16*(TrancheA*IF(1-VerifLag=Pipeline!$I17,RampV1,IF(1-VerifLag=Pipeline!$I17+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I17+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I17,RampV1,IF(1-VerifLag-1=Pipeline!$I17+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I17+2,1-RampV2,0))))</f>
-        <v>54753.070754717</v>
+        <v>49775.5188679245</v>
       </c>
       <c r="H16" s="47" t="n">
         <f aca="false">$C16*$E16*(TrancheA*IF(2-VerifLag=Pipeline!$I17,RampV1,IF(2-VerifLag=Pipeline!$I17+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I17+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I17,RampV1,IF(2-VerifLag-1=Pipeline!$I17+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I17+2,1-RampV2,0))))</f>
-        <v>50842.1371293801</v>
+        <v>46220.1246630728</v>
       </c>
       <c r="I16" s="47" t="n">
         <f aca="false">$C16*$E16*(TrancheA*IF(3-VerifLag=Pipeline!$I17,RampV1,IF(3-VerifLag=Pipeline!$I17+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I17+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I17,RampV1,IF(3-VerifLag-1=Pipeline!$I17+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I17+2,1-RampV2,0))))</f>
-        <v>20858.3126684636</v>
+        <v>18962.102425876</v>
       </c>
       <c r="J16" s="47" t="n">
         <f aca="false">$C16*$E16*(TrancheA*IF(4-VerifLag=Pipeline!$I17,RampV1,IF(4-VerifLag=Pipeline!$I17+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I17+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I17,RampV1,IF(4-VerifLag-1=Pipeline!$I17+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I17+2,1-RampV2,0))))</f>
-        <v>3910.93362533693</v>
+        <v>3555.39420485175</v>
       </c>
       <c r="K16" s="47" t="n">
         <f aca="false">$C16*$E16*(TrancheA*IF(5-VerifLag=Pipeline!$I17,RampV1,IF(5-VerifLag=Pipeline!$I17+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I17+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I17,RampV1,IF(5-VerifLag-1=Pipeline!$I17+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I17+2,1-RampV2,0))))</f>
@@ -12455,7 +12455,7 @@
       </c>
       <c r="Q16" s="48" t="n">
         <f aca="false">SUM(G16:P16)</f>
-        <v>130364.454177898</v>
+        <v>118513.140161725</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12468,11 +12468,11 @@
       </c>
       <c r="C17" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18*'Eligibility &amp; Scoring'!$U18</f>
-        <v>122718.75</v>
+        <v>111562.5</v>
       </c>
       <c r="D17" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18-C17</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
       <c r="E17" s="29" t="n">
         <f aca="false">IF(C17+D17=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H18),1))</f>
@@ -12480,7 +12480,7 @@
       </c>
       <c r="F17" s="28" t="n">
         <f aca="false">C17*E17</f>
-        <v>110446.875</v>
+        <v>100406.25</v>
       </c>
       <c r="G17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(1-VerifLag=Pipeline!$I18,RampV1,IF(1-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I18,RampV1,IF(1-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
@@ -12488,19 +12488,19 @@
       </c>
       <c r="H17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(2-VerifLag=Pipeline!$I18,RampV1,IF(2-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I18,RampV1,IF(2-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
-        <v>46387.6875</v>
+        <v>42170.625</v>
       </c>
       <c r="I17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(3-VerifLag=Pipeline!$I18,RampV1,IF(3-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I18,RampV1,IF(3-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
-        <v>43074.28125</v>
+        <v>39158.4375</v>
       </c>
       <c r="J17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(4-VerifLag=Pipeline!$I18,RampV1,IF(4-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I18,RampV1,IF(4-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
-        <v>17671.5</v>
+        <v>16065</v>
       </c>
       <c r="K17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(5-VerifLag=Pipeline!$I18,RampV1,IF(5-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I18,RampV1,IF(5-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
-        <v>3313.40625</v>
+        <v>3012.1875</v>
       </c>
       <c r="L17" s="47" t="n">
         <f aca="false">$C17*$E17*(TrancheA*IF(6-VerifLag=Pipeline!$I18,RampV1,IF(6-VerifLag=Pipeline!$I18+1,RampV2-RampV1,IF(6-VerifLag=Pipeline!$I18+2,1-RampV2,0)))+(1-TrancheA)*IF(6-VerifLag-1=Pipeline!$I18,RampV1,IF(6-VerifLag-1=Pipeline!$I18+1,RampV2-RampV1,IF(6-VerifLag-1=Pipeline!$I18+2,1-RampV2,0))))</f>
@@ -12524,7 +12524,7 @@
       </c>
       <c r="Q17" s="48" t="n">
         <f aca="false">SUM(G17:P17)</f>
-        <v>110446.875</v>
+        <v>100406.25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12606,11 +12606,11 @@
       </c>
       <c r="C19" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20*'Eligibility &amp; Scoring'!$U20</f>
-        <v>39784.3839541547</v>
+        <v>36167.6217765043</v>
       </c>
       <c r="D19" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20-C19</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
       <c r="E19" s="29" t="n">
         <f aca="false">IF(C19+D19=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H20),1))</f>
@@ -12618,7 +12618,7 @@
       </c>
       <c r="F19" s="28" t="n">
         <f aca="false">C19*E19</f>
-        <v>37795.164756447</v>
+        <v>34359.2406876791</v>
       </c>
       <c r="G19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(1-VerifLag=Pipeline!$I20,RampV1,IF(1-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(1-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(1-VerifLag-1=Pipeline!$I20,RampV1,IF(1-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(1-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
@@ -12626,19 +12626,19 @@
       </c>
       <c r="H19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(2-VerifLag=Pipeline!$I20,RampV1,IF(2-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(2-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(2-VerifLag-1=Pipeline!$I20,RampV1,IF(2-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(2-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
-        <v>15873.9691977077</v>
+        <v>14430.8810888252</v>
       </c>
       <c r="I19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(3-VerifLag=Pipeline!$I20,RampV1,IF(3-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(3-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(3-VerifLag-1=Pipeline!$I20,RampV1,IF(3-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(3-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
-        <v>14740.1142550143</v>
+        <v>13400.1038681948</v>
       </c>
       <c r="J19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(4-VerifLag=Pipeline!$I20,RampV1,IF(4-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(4-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(4-VerifLag-1=Pipeline!$I20,RampV1,IF(4-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(4-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
-        <v>6047.22636103152</v>
+        <v>5497.47851002865</v>
       </c>
       <c r="K19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(5-VerifLag=Pipeline!$I20,RampV1,IF(5-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(5-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(5-VerifLag-1=Pipeline!$I20,RampV1,IF(5-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(5-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
-        <v>1133.85494269341</v>
+        <v>1030.77722063037</v>
       </c>
       <c r="L19" s="47" t="n">
         <f aca="false">$C19*$E19*(TrancheA*IF(6-VerifLag=Pipeline!$I20,RampV1,IF(6-VerifLag=Pipeline!$I20+1,RampV2-RampV1,IF(6-VerifLag=Pipeline!$I20+2,1-RampV2,0)))+(1-TrancheA)*IF(6-VerifLag-1=Pipeline!$I20,RampV1,IF(6-VerifLag-1=Pipeline!$I20+1,RampV2-RampV1,IF(6-VerifLag-1=Pipeline!$I20+2,1-RampV2,0))))</f>
@@ -12662,7 +12662,7 @@
       </c>
       <c r="Q19" s="48" t="n">
         <f aca="false">SUM(G19:P19)</f>
-        <v>37795.164756447</v>
+        <v>34359.2406876791</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13430,35 +13430,35 @@
       </c>
       <c r="C31" s="43" t="n">
         <f aca="false">SUM(C6:C30)</f>
-        <v>823387.761378275</v>
+        <v>753310.82158811</v>
       </c>
       <c r="D31" s="43" t="n">
         <f aca="false">SUM(D6:D30)</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
       <c r="F31" s="43" t="n">
         <f aca="false">SUM(F6:F30)</f>
-        <v>774834.812479654</v>
+        <v>708694.127828577</v>
       </c>
       <c r="G31" s="43" t="n">
         <f aca="false">SUM(G6:G30)</f>
-        <v>156598.271110424</v>
+        <v>142362.06464584</v>
       </c>
       <c r="H31" s="43" t="n">
         <f aca="false">SUM(H6:H30)</f>
-        <v>314245.030447853</v>
+        <v>287482.814784728</v>
       </c>
       <c r="I31" s="43" t="n">
         <f aca="false">SUM(I6:I30)</f>
-        <v>216429.380782786</v>
+        <v>198430.531594709</v>
       </c>
       <c r="J31" s="43" t="n">
         <f aca="false">SUM(J6:J30)</f>
-        <v>75502.676557804</v>
+        <v>69326.6118717172</v>
       </c>
       <c r="K31" s="43" t="n">
         <f aca="false">SUM(K6:K30)</f>
-        <v>12059.4535807879</v>
+        <v>11092.1049315831</v>
       </c>
       <c r="L31" s="43" t="n">
         <f aca="false">SUM(L6:L30)</f>
@@ -13482,7 +13482,7 @@
       </c>
       <c r="Q31" s="43" t="n">
         <f aca="false">SUM(Q6:Q30)</f>
-        <v>774834.812479654</v>
+        <v>708694.127828577</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13579,11 +13579,11 @@
       </c>
       <c r="C35" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7*'Eligibility &amp; Scoring'!$U7</f>
-        <v>121856.557377049</v>
+        <v>110778.68852459</v>
       </c>
       <c r="D35" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7-C35</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
       <c r="E35" s="29" t="n">
         <f aca="false">IF(C35+D35=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H7),1))</f>
@@ -13591,11 +13591,11 @@
       </c>
       <c r="F35" s="28" t="n">
         <f aca="false">D35</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
       <c r="G35" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I7,$D35,0)</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
       <c r="H35" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I7,$D35,0)</f>
@@ -13635,7 +13635,7 @@
       </c>
       <c r="Q35" s="48" t="n">
         <f aca="false">SUM(G35:P35)</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13648,11 +13648,11 @@
       </c>
       <c r="C36" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8*'Eligibility &amp; Scoring'!$U8</f>
-        <v>82500</v>
+        <v>32871.09375</v>
       </c>
       <c r="D36" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8-C36</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
       <c r="E36" s="29" t="n">
         <f aca="false">IF(C36+D36=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H8),1))</f>
@@ -13660,7 +13660,7 @@
       </c>
       <c r="F36" s="28" t="n">
         <f aca="false">D36</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
       <c r="G36" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I8,$D36,0)</f>
@@ -13668,7 +13668,7 @@
       </c>
       <c r="H36" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I8,$D36,0)</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
       <c r="I36" s="47" t="n">
         <f aca="false">IF(3=Pipeline!$I8,$D36,0)</f>
@@ -13704,7 +13704,7 @@
       </c>
       <c r="Q36" s="48" t="n">
         <f aca="false">SUM(G36:P36)</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13717,11 +13717,11 @@
       </c>
       <c r="C37" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9*'Eligibility &amp; Scoring'!$U9</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
       <c r="D37" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9-C37</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
       <c r="E37" s="29" t="n">
         <f aca="false">IF(C37+D37=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H9),1))</f>
@@ -13729,11 +13729,11 @@
       </c>
       <c r="F37" s="28" t="n">
         <f aca="false">D37</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
       <c r="G37" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I9,$D37,0)</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
       <c r="H37" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I9,$D37,0)</f>
@@ -13773,7 +13773,7 @@
       </c>
       <c r="Q37" s="48" t="n">
         <f aca="false">SUM(G37:P37)</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14062,11 +14062,11 @@
       </c>
       <c r="C42" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14*'Eligibility &amp; Scoring'!$U14</f>
-        <v>123400.176678445</v>
+        <v>112181.978798587</v>
       </c>
       <c r="D42" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14-C42</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
       <c r="E42" s="29" t="n">
         <f aca="false">IF(C42+D42=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H14),1))</f>
@@ -14074,7 +14074,7 @@
       </c>
       <c r="F42" s="28" t="n">
         <f aca="false">D42</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
       <c r="G42" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I14,$D42,0)</f>
@@ -14082,7 +14082,7 @@
       </c>
       <c r="H42" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I14,$D42,0)</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
       <c r="I42" s="47" t="n">
         <f aca="false">IF(3=Pipeline!$I14,$D42,0)</f>
@@ -14118,7 +14118,7 @@
       </c>
       <c r="Q42" s="48" t="n">
         <f aca="false">SUM(G42:P42)</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14131,11 +14131,11 @@
       </c>
       <c r="C43" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15*'Eligibility &amp; Scoring'!$U15</f>
-        <v>69177.3093614383</v>
+        <v>109793.862368258</v>
       </c>
       <c r="D43" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15-C43</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
       <c r="E43" s="29" t="n">
         <f aca="false">IF(C43+D43=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H15),1))</f>
@@ -14143,7 +14143,7 @@
       </c>
       <c r="F43" s="28" t="n">
         <f aca="false">D43</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
       <c r="G43" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I15,$D43,0)</f>
@@ -14151,7 +14151,7 @@
       </c>
       <c r="H43" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I15,$D43,0)</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
       <c r="I43" s="47" t="n">
         <f aca="false">IF(3=Pipeline!$I15,$D43,0)</f>
@@ -14187,7 +14187,7 @@
       </c>
       <c r="Q43" s="48" t="n">
         <f aca="false">SUM(G43:P43)</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14269,11 +14269,11 @@
       </c>
       <c r="C45" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17*'Eligibility &amp; Scoring'!$U17</f>
-        <v>137225.741239892</v>
+        <v>124750.673854447</v>
       </c>
       <c r="D45" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17-C45</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
       <c r="E45" s="29" t="n">
         <f aca="false">IF(C45+D45=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H17),1))</f>
@@ -14281,11 +14281,11 @@
       </c>
       <c r="F45" s="28" t="n">
         <f aca="false">D45</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
       <c r="G45" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I17,$D45,0)</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
       <c r="H45" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I17,$D45,0)</f>
@@ -14325,7 +14325,7 @@
       </c>
       <c r="Q45" s="48" t="n">
         <f aca="false">SUM(G45:P45)</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14338,11 +14338,11 @@
       </c>
       <c r="C46" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18*'Eligibility &amp; Scoring'!$U18</f>
-        <v>122718.75</v>
+        <v>111562.5</v>
       </c>
       <c r="D46" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18-C46</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
       <c r="E46" s="29" t="n">
         <f aca="false">IF(C46+D46=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H18),1))</f>
@@ -14350,7 +14350,7 @@
       </c>
       <c r="F46" s="28" t="n">
         <f aca="false">D46</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
       <c r="G46" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I18,$D46,0)</f>
@@ -14358,7 +14358,7 @@
       </c>
       <c r="H46" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I18,$D46,0)</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
       <c r="I46" s="47" t="n">
         <f aca="false">IF(3=Pipeline!$I18,$D46,0)</f>
@@ -14394,7 +14394,7 @@
       </c>
       <c r="Q46" s="48" t="n">
         <f aca="false">SUM(G46:P46)</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -14476,11 +14476,11 @@
       </c>
       <c r="C48" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20*'Eligibility &amp; Scoring'!$U20</f>
-        <v>39784.3839541547</v>
+        <v>36167.6217765043</v>
       </c>
       <c r="D48" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20-C48</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
       <c r="E48" s="29" t="n">
         <f aca="false">IF(C48+D48=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H20),1))</f>
@@ -14488,7 +14488,7 @@
       </c>
       <c r="F48" s="28" t="n">
         <f aca="false">D48</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
       <c r="G48" s="47" t="n">
         <f aca="false">IF(1=Pipeline!$I20,$D48,0)</f>
@@ -14496,7 +14496,7 @@
       </c>
       <c r="H48" s="47" t="n">
         <f aca="false">IF(2=Pipeline!$I20,$D48,0)</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
       <c r="I48" s="47" t="n">
         <f aca="false">IF(3=Pipeline!$I20,$D48,0)</f>
@@ -14532,7 +14532,7 @@
       </c>
       <c r="Q48" s="48" t="n">
         <f aca="false">SUM(G48:P48)</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15300,23 +15300,23 @@
       </c>
       <c r="C60" s="43" t="n">
         <f aca="false">SUM(C35:C59)</f>
-        <v>823387.761378275</v>
+        <v>753310.82158811</v>
       </c>
       <c r="D60" s="43" t="n">
         <f aca="false">SUM(D35:D59)</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
       <c r="F60" s="43" t="n">
         <f aca="false">SUM(F35:F59)</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
       <c r="G60" s="43" t="n">
         <f aca="false">SUM(G35:G59)</f>
-        <v>876442.858615763</v>
+        <v>796766.235105239</v>
       </c>
       <c r="H60" s="43" t="n">
         <f aca="false">SUM(H35:H59)</f>
-        <v>1105169.38000596</v>
+        <v>999922.943306651</v>
       </c>
       <c r="I60" s="43" t="n">
         <f aca="false">SUM(I35:I59)</f>
@@ -15352,7 +15352,7 @@
       </c>
       <c r="Q60" s="43" t="n">
         <f aca="false">SUM(Q35:Q59)</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15449,11 +15449,11 @@
       </c>
       <c r="C64" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7*'Eligibility &amp; Scoring'!$U7</f>
-        <v>121856.557377049</v>
+        <v>110778.68852459</v>
       </c>
       <c r="D64" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK7-C64</f>
-        <v>298893.442622951</v>
+        <v>271721.31147541</v>
       </c>
       <c r="E64" s="29" t="n">
         <f aca="false">IF(C64+D64=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H7),1))</f>
@@ -15461,23 +15461,23 @@
       </c>
       <c r="F64" s="28" t="n">
         <f aca="false">C64*E64+D64</f>
-        <v>414657.172131148</v>
+        <v>376961.065573771</v>
       </c>
       <c r="G64" s="47" t="n">
         <f aca="false">G6+G35</f>
-        <v>347514.209016393</v>
+        <v>315922.008196721</v>
       </c>
       <c r="H64" s="47" t="n">
         <f aca="false">H6+H35</f>
-        <v>45147.8545081967</v>
+        <v>41043.5040983607</v>
       </c>
       <c r="I64" s="47" t="n">
         <f aca="false">I6+I35</f>
-        <v>18522.1967213115</v>
+        <v>16838.3606557377</v>
       </c>
       <c r="J64" s="47" t="n">
         <f aca="false">J6+J35</f>
-        <v>3472.9118852459</v>
+        <v>3157.19262295082</v>
       </c>
       <c r="K64" s="47" t="n">
         <f aca="false">K6+K35</f>
@@ -15505,7 +15505,7 @@
       </c>
       <c r="Q64" s="48" t="n">
         <f aca="false">SUM(G64:P64)</f>
-        <v>414657.172131148</v>
+        <v>376961.065573771</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15518,11 +15518,11 @@
       </c>
       <c r="C65" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8*'Eligibility &amp; Scoring'!$U8</f>
-        <v>82500</v>
+        <v>32871.09375</v>
       </c>
       <c r="D65" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK8-C65</f>
-        <v>237500</v>
+        <v>94628.90625</v>
       </c>
       <c r="E65" s="29" t="n">
         <f aca="false">IF(C65+D65=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H8),1))</f>
@@ -15530,7 +15530,7 @@
       </c>
       <c r="F65" s="28" t="n">
         <f aca="false">C65*E65+D65</f>
-        <v>311750</v>
+        <v>124212.890625</v>
       </c>
       <c r="G65" s="47" t="n">
         <f aca="false">G7+G36</f>
@@ -15538,19 +15538,19 @@
       </c>
       <c r="H65" s="47" t="n">
         <f aca="false">H7+H36</f>
-        <v>268685</v>
+        <v>107054.1796875</v>
       </c>
       <c r="I65" s="47" t="n">
         <f aca="false">I7+I36</f>
-        <v>28957.5</v>
+        <v>11537.75390625</v>
       </c>
       <c r="J65" s="47" t="n">
         <f aca="false">J7+J36</f>
-        <v>11880</v>
+        <v>4733.4375</v>
       </c>
       <c r="K65" s="47" t="n">
         <f aca="false">K7+K36</f>
-        <v>2227.5</v>
+        <v>887.51953125</v>
       </c>
       <c r="L65" s="47" t="n">
         <f aca="false">L7+L36</f>
@@ -15574,7 +15574,7 @@
       </c>
       <c r="Q65" s="48" t="n">
         <f aca="false">SUM(G65:P65)</f>
-        <v>311750</v>
+        <v>124212.890625</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15587,11 +15587,11 @@
       </c>
       <c r="C66" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9*'Eligibility &amp; Scoring'!$U9</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
       <c r="D66" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK9-C66</f>
-        <v>294025.157232704</v>
+        <v>267295.597484277</v>
       </c>
       <c r="E66" s="29" t="n">
         <f aca="false">IF(C66+D66=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H9),1))</f>
@@ -15599,23 +15599,23 @@
       </c>
       <c r="F66" s="28" t="n">
         <f aca="false">C66*E66+D66</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
       <c r="G66" s="47" t="n">
         <f aca="false">G8+G37</f>
-        <v>347249.591194969</v>
+        <v>315681.446540881</v>
       </c>
       <c r="H66" s="47" t="n">
         <f aca="false">H8+H37</f>
-        <v>49422.6886792453</v>
+        <v>44929.7169811321</v>
       </c>
       <c r="I66" s="47" t="n">
         <f aca="false">I8+I37</f>
-        <v>20275.9748427673</v>
+        <v>18432.7044025157</v>
       </c>
       <c r="J66" s="47" t="n">
         <f aca="false">J8+J37</f>
-        <v>3801.74528301887</v>
+        <v>3456.1320754717</v>
       </c>
       <c r="K66" s="47" t="n">
         <f aca="false">K8+K37</f>
@@ -15643,7 +15643,7 @@
       </c>
       <c r="Q66" s="48" t="n">
         <f aca="false">SUM(G66:P66)</f>
-        <v>420750</v>
+        <v>382500</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -15932,11 +15932,11 @@
       </c>
       <c r="C71" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14*'Eligibility &amp; Scoring'!$U14</f>
-        <v>123400.176678445</v>
+        <v>112181.978798587</v>
       </c>
       <c r="D71" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK14-C71</f>
-        <v>297349.823321555</v>
+        <v>270318.021201413</v>
       </c>
       <c r="E71" s="29" t="n">
         <f aca="false">IF(C71+D71=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H14),1))</f>
@@ -15944,7 +15944,7 @@
       </c>
       <c r="F71" s="28" t="n">
         <f aca="false">C71*E71+D71</f>
-        <v>414579.991166078</v>
+        <v>376890.901060071</v>
       </c>
       <c r="G71" s="47" t="n">
         <f aca="false">G13+G42</f>
@@ -15952,19 +15952,19 @@
       </c>
       <c r="H71" s="47" t="n">
         <f aca="false">H13+H42</f>
-        <v>346586.493816254</v>
+        <v>315078.630742049</v>
       </c>
       <c r="I71" s="47" t="n">
         <f aca="false">I13+I42</f>
-        <v>45719.765459364</v>
+        <v>41563.4231448763</v>
       </c>
       <c r="J71" s="47" t="n">
         <f aca="false">J13+J42</f>
-        <v>18756.8268551237</v>
+        <v>17051.6607773852</v>
       </c>
       <c r="K71" s="47" t="n">
         <f aca="false">K13+K42</f>
-        <v>3516.90503533569</v>
+        <v>3197.18639575972</v>
       </c>
       <c r="L71" s="47" t="n">
         <f aca="false">L13+L42</f>
@@ -15988,7 +15988,7 @@
       </c>
       <c r="Q71" s="48" t="n">
         <f aca="false">SUM(G71:P71)</f>
-        <v>414579.991166078</v>
+        <v>376890.901060071</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16001,11 +16001,11 @@
       </c>
       <c r="C72" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15*'Eligibility &amp; Scoring'!$U15</f>
-        <v>69177.3093614383</v>
+        <v>109793.862368258</v>
       </c>
       <c r="D72" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK15-C72</f>
-        <v>171822.690638562</v>
+        <v>272706.137631742</v>
       </c>
       <c r="E72" s="29" t="n">
         <f aca="false">IF(C72+D72=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H15),1))</f>
@@ -16013,7 +16013,7 @@
       </c>
       <c r="F72" s="28" t="n">
         <f aca="false">C72*E72+D72</f>
-        <v>234082.269063856</v>
+        <v>371520.613763174</v>
       </c>
       <c r="G72" s="47" t="n">
         <f aca="false">G14+G43</f>
@@ -16021,19 +16021,19 @@
       </c>
       <c r="H72" s="47" t="n">
         <f aca="false">H14+H43</f>
-        <v>197971.713577185</v>
+        <v>314208.217606944</v>
       </c>
       <c r="I72" s="47" t="n">
         <f aca="false">I14+I43</f>
-        <v>24281.2355858648</v>
+        <v>38537.6456912585</v>
       </c>
       <c r="J72" s="47" t="n">
         <f aca="false">J14+J43</f>
-        <v>9961.53254804712</v>
+        <v>15810.3161810291</v>
       </c>
       <c r="K72" s="47" t="n">
         <f aca="false">K14+K43</f>
-        <v>1867.78735275883</v>
+        <v>2964.43428394296</v>
       </c>
       <c r="L72" s="47" t="n">
         <f aca="false">L14+L43</f>
@@ -16057,7 +16057,7 @@
       </c>
       <c r="Q72" s="48" t="n">
         <f aca="false">SUM(G72:P72)</f>
-        <v>234082.269063856</v>
+        <v>371520.613763174</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16139,11 +16139,11 @@
       </c>
       <c r="C74" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17*'Eligibility &amp; Scoring'!$U17</f>
-        <v>137225.741239892</v>
+        <v>124750.673854447</v>
       </c>
       <c r="D74" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK17-C74</f>
-        <v>283524.258760108</v>
+        <v>257749.326145553</v>
       </c>
       <c r="E74" s="29" t="n">
         <f aca="false">IF(C74+D74=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H17),1))</f>
@@ -16151,23 +16151,23 @@
       </c>
       <c r="F74" s="28" t="n">
         <f aca="false">C74*E74+D74</f>
-        <v>413888.712938005</v>
+        <v>376262.466307278</v>
       </c>
       <c r="G74" s="47" t="n">
         <f aca="false">G16+G45</f>
-        <v>338277.329514825</v>
+        <v>307524.845013477</v>
       </c>
       <c r="H74" s="47" t="n">
         <f aca="false">H16+H45</f>
-        <v>50842.1371293801</v>
+        <v>46220.1246630728</v>
       </c>
       <c r="I74" s="47" t="n">
         <f aca="false">I16+I45</f>
-        <v>20858.3126684636</v>
+        <v>18962.102425876</v>
       </c>
       <c r="J74" s="47" t="n">
         <f aca="false">J16+J45</f>
-        <v>3910.93362533693</v>
+        <v>3555.39420485175</v>
       </c>
       <c r="K74" s="47" t="n">
         <f aca="false">K16+K45</f>
@@ -16195,7 +16195,7 @@
       </c>
       <c r="Q74" s="48" t="n">
         <f aca="false">SUM(G74:P74)</f>
-        <v>413888.712938005</v>
+        <v>376262.466307278</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16208,11 +16208,11 @@
       </c>
       <c r="C75" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18*'Eligibility &amp; Scoring'!$U18</f>
-        <v>122718.75</v>
+        <v>111562.5</v>
       </c>
       <c r="D75" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK18-C75</f>
-        <v>298031.25</v>
+        <v>270937.5</v>
       </c>
       <c r="E75" s="29" t="n">
         <f aca="false">IF(C75+D75=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H18),1))</f>
@@ -16220,7 +16220,7 @@
       </c>
       <c r="F75" s="28" t="n">
         <f aca="false">C75*E75+D75</f>
-        <v>408478.125</v>
+        <v>371343.75</v>
       </c>
       <c r="G75" s="47" t="n">
         <f aca="false">G17+G46</f>
@@ -16228,19 +16228,19 @@
       </c>
       <c r="H75" s="47" t="n">
         <f aca="false">H17+H46</f>
-        <v>344418.9375</v>
+        <v>313108.125</v>
       </c>
       <c r="I75" s="47" t="n">
         <f aca="false">I17+I46</f>
-        <v>43074.28125</v>
+        <v>39158.4375</v>
       </c>
       <c r="J75" s="47" t="n">
         <f aca="false">J17+J46</f>
-        <v>17671.5</v>
+        <v>16065</v>
       </c>
       <c r="K75" s="47" t="n">
         <f aca="false">K17+K46</f>
-        <v>3313.40625</v>
+        <v>3012.1875</v>
       </c>
       <c r="L75" s="47" t="n">
         <f aca="false">L17+L46</f>
@@ -16264,7 +16264,7 @@
       </c>
       <c r="Q75" s="48" t="n">
         <f aca="false">SUM(G75:P75)</f>
-        <v>408478.125</v>
+        <v>371343.75</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16346,11 +16346,11 @@
       </c>
       <c r="C77" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20*'Eligibility &amp; Scoring'!$U20</f>
-        <v>39784.3839541547</v>
+        <v>36167.6217765043</v>
       </c>
       <c r="D77" s="28" t="n">
         <f aca="false">'Eligibility &amp; Scoring'!$AK20-C77</f>
-        <v>100465.616045845</v>
+        <v>91332.3782234957</v>
       </c>
       <c r="E77" s="29" t="n">
         <f aca="false">IF(C77+D77=0,0,IFERROR(INDEX('Fund Parameters'!$B$74:$B$78,Pipeline!$H20),1))</f>
@@ -16358,7 +16358,7 @@
       </c>
       <c r="F77" s="28" t="n">
         <f aca="false">C77*E77+D77</f>
-        <v>138260.780802292</v>
+        <v>125691.618911175</v>
       </c>
       <c r="G77" s="47" t="n">
         <f aca="false">G19+G48</f>
@@ -16366,19 +16366,19 @@
       </c>
       <c r="H77" s="47" t="n">
         <f aca="false">H19+H48</f>
-        <v>116339.585243553</v>
+        <v>105763.259312321</v>
       </c>
       <c r="I77" s="47" t="n">
         <f aca="false">I19+I48</f>
-        <v>14740.1142550143</v>
+        <v>13400.1038681948</v>
       </c>
       <c r="J77" s="47" t="n">
         <f aca="false">J19+J48</f>
-        <v>6047.22636103152</v>
+        <v>5497.47851002865</v>
       </c>
       <c r="K77" s="47" t="n">
         <f aca="false">K19+K48</f>
-        <v>1133.85494269341</v>
+        <v>1030.77722063037</v>
       </c>
       <c r="L77" s="47" t="n">
         <f aca="false">L19+L48</f>
@@ -16402,7 +16402,7 @@
       </c>
       <c r="Q77" s="48" t="n">
         <f aca="false">SUM(G77:P77)</f>
-        <v>138260.780802292</v>
+        <v>125691.618911175</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17170,35 +17170,35 @@
       </c>
       <c r="C89" s="43" t="n">
         <f aca="false">SUM(C64:C88)</f>
-        <v>823387.761378275</v>
+        <v>753310.82158811</v>
       </c>
       <c r="D89" s="43" t="n">
         <f aca="false">SUM(D64:D88)</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
       <c r="F89" s="43" t="n">
         <f aca="false">SUM(F64:F88)</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="G89" s="43" t="n">
         <f aca="false">SUM(G64:G88)</f>
-        <v>1033041.12972619</v>
+        <v>939128.299751079</v>
       </c>
       <c r="H89" s="43" t="n">
         <f aca="false">SUM(H64:H88)</f>
-        <v>1419414.41045381</v>
+        <v>1287405.75809138</v>
       </c>
       <c r="I89" s="43" t="n">
         <f aca="false">SUM(I64:I88)</f>
-        <v>216429.380782786</v>
+        <v>198430.531594709</v>
       </c>
       <c r="J89" s="43" t="n">
         <f aca="false">SUM(J64:J88)</f>
-        <v>75502.676557804</v>
+        <v>69326.6118717172</v>
       </c>
       <c r="K89" s="43" t="n">
         <f aca="false">SUM(K64:K88)</f>
-        <v>12059.4535807879</v>
+        <v>11092.1049315831</v>
       </c>
       <c r="L89" s="43" t="n">
         <f aca="false">SUM(L64:L88)</f>
@@ -17222,7 +17222,7 @@
       </c>
       <c r="Q89" s="43" t="n">
         <f aca="false">SUM(Q64:Q88)</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17252,23 +17252,23 @@
       </c>
       <c r="G93" s="47" t="n">
         <f aca="false">G89</f>
-        <v>1033041.12972619</v>
+        <v>939128.299751079</v>
       </c>
       <c r="H93" s="47" t="n">
         <f aca="false">H89</f>
-        <v>1419414.41045381</v>
+        <v>1287405.75809138</v>
       </c>
       <c r="I93" s="47" t="n">
         <f aca="false">I89</f>
-        <v>216429.380782786</v>
+        <v>198430.531594709</v>
       </c>
       <c r="J93" s="47" t="n">
         <f aca="false">J89</f>
-        <v>75502.676557804</v>
+        <v>69326.6118717172</v>
       </c>
       <c r="K93" s="47" t="n">
         <f aca="false">K89</f>
-        <v>12059.4535807879</v>
+        <v>11092.1049315831</v>
       </c>
       <c r="L93" s="47" t="n">
         <f aca="false">L89</f>
@@ -17297,43 +17297,43 @@
       </c>
       <c r="G94" s="47" t="n">
         <f aca="false">G93</f>
-        <v>1033041.12972619</v>
+        <v>939128.299751079</v>
       </c>
       <c r="H94" s="47" t="n">
         <f aca="false">G94+H93</f>
-        <v>2452455.54018</v>
+        <v>2226534.05784246</v>
       </c>
       <c r="I94" s="47" t="n">
         <f aca="false">H94+I93</f>
-        <v>2668884.92096279</v>
+        <v>2424964.58943717</v>
       </c>
       <c r="J94" s="47" t="n">
         <f aca="false">I94+J93</f>
-        <v>2744387.59752059</v>
+        <v>2494291.20130888</v>
       </c>
       <c r="K94" s="47" t="n">
         <f aca="false">J94+K93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="L94" s="47" t="n">
         <f aca="false">K94+L93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="M94" s="47" t="n">
         <f aca="false">L94+M93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="N94" s="47" t="n">
         <f aca="false">M94+N93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="O94" s="47" t="n">
         <f aca="false">N94+O93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="P94" s="47" t="n">
         <f aca="false">O94+P93</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17342,43 +17342,43 @@
       </c>
       <c r="G95" s="48" t="n">
         <f aca="false">Available-G94</f>
-        <v>1516958.87027381</v>
+        <v>1610871.70024892</v>
       </c>
       <c r="H95" s="48" t="n">
         <f aca="false">Available-H94</f>
-        <v>97544.4598199986</v>
+        <v>323465.942157541</v>
       </c>
       <c r="I95" s="48" t="n">
         <f aca="false">Available-I94</f>
-        <v>-118884.920962787</v>
+        <v>125035.410562832</v>
       </c>
       <c r="J95" s="48" t="n">
         <f aca="false">Available-J94</f>
-        <v>-194387.597520591</v>
+        <v>55708.7986911153</v>
       </c>
       <c r="K95" s="48" t="n">
         <f aca="false">Available-K94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="L95" s="48" t="n">
         <f aca="false">Available-L94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="M95" s="48" t="n">
         <f aca="false">Available-M94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="N95" s="48" t="n">
         <f aca="false">Available-N94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="O95" s="48" t="n">
         <f aca="false">Available-O94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="P95" s="48" t="n">
         <f aca="false">Available-P94</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17387,43 +17387,43 @@
       </c>
       <c r="G96" s="47" t="n">
         <f aca="false">TotalAllocated-G94</f>
-        <v>1771958.87027381</v>
+        <v>1610871.70024892</v>
       </c>
       <c r="H96" s="47" t="n">
         <f aca="false">TotalAllocated-H94</f>
-        <v>352544.459819999</v>
+        <v>323465.942157541</v>
       </c>
       <c r="I96" s="47" t="n">
         <f aca="false">TotalAllocated-I94</f>
-        <v>136115.079037213</v>
+        <v>125035.410562832</v>
       </c>
       <c r="J96" s="47" t="n">
         <f aca="false">TotalAllocated-J94</f>
-        <v>60612.4024794092</v>
+        <v>55708.7986911153</v>
       </c>
       <c r="K96" s="47" t="n">
         <f aca="false">TotalAllocated-K94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="L96" s="47" t="n">
         <f aca="false">TotalAllocated-L94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="M96" s="47" t="n">
         <f aca="false">TotalAllocated-M94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="N96" s="47" t="n">
         <f aca="false">TotalAllocated-N94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="O96" s="47" t="n">
         <f aca="false">TotalAllocated-O94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
       <c r="P96" s="47" t="n">
         <f aca="false">TotalAllocated-P94</f>
-        <v>48552.9488986214</v>
+        <v>44616.6937595322</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="C97" s="48" t="n">
         <f aca="false">SUM(C6:C30)-Q31</f>
-        <v>48552.9488986209</v>
+        <v>44616.6937595323</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17441,7 +17441,7 @@
       </c>
       <c r="C98" s="48" t="n">
         <f aca="false">MIN(G95:P95)</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
     </row>
   </sheetData>
@@ -17550,7 +17550,7 @@
       </c>
       <c r="D7" s="36" t="n">
         <f aca="false">Disbursements!$C$6</f>
-        <v>121856.557377049</v>
+        <v>110778.68852459</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>1048</v>
@@ -17569,12 +17569,12 @@
       </c>
       <c r="I7" s="28" t="n">
         <f aca="false">IFERROR(MIN(D7,E7/C7*D7),0)</f>
-        <v>118245.992714025</v>
+        <v>107496.35701275</v>
       </c>
       <c r="J7" s="13"/>
       <c r="K7" s="28" t="n">
         <f aca="false">MAX(0,I7*TrancheA-J7)</f>
-        <v>82772.1948998178</v>
+        <v>75247.4499089253</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17591,7 +17591,7 @@
       </c>
       <c r="D8" s="36" t="n">
         <f aca="false">Disbursements!$C$7</f>
-        <v>82500</v>
+        <v>32871.09375</v>
       </c>
       <c r="E8" s="22" t="n">
         <v>487</v>
@@ -17610,12 +17610,12 @@
       </c>
       <c r="I8" s="28" t="n">
         <f aca="false">IFERROR(MIN(D8,E8/C8*D8),0)</f>
-        <v>57726.2931034483</v>
+        <v>23000.3199084052</v>
       </c>
       <c r="J8" s="13"/>
       <c r="K8" s="28" t="n">
         <f aca="false">MAX(0,I8*TrancheA-J8)</f>
-        <v>40408.4051724138</v>
+        <v>16100.2239358836</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17632,7 +17632,7 @@
       </c>
       <c r="D9" s="36" t="n">
         <f aca="false">Disbursements!$C$8</f>
-        <v>126724.842767296</v>
+        <v>115204.402515723</v>
       </c>
       <c r="E9" s="22" t="n">
         <v>1371</v>
@@ -17651,12 +17651,12 @@
       </c>
       <c r="I9" s="28" t="n">
         <f aca="false">IFERROR(MIN(D9,E9/C9*D9),0)</f>
-        <v>101365.087184342</v>
+        <v>92150.0792584928</v>
       </c>
       <c r="J9" s="13"/>
       <c r="K9" s="28" t="n">
         <f aca="false">MAX(0,I9*TrancheA-J9)</f>
-        <v>70955.5610290394</v>
+        <v>64505.0554809449</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17837,7 +17837,7 @@
       </c>
       <c r="D14" s="36" t="n">
         <f aca="false">Disbursements!$C$13</f>
-        <v>123400.176678445</v>
+        <v>112181.978798587</v>
       </c>
       <c r="E14" s="22" t="n">
         <v>745</v>
@@ -17856,12 +17856,12 @@
       </c>
       <c r="I14" s="28" t="n">
         <f aca="false">IFERROR(MIN(D14,E14/C14*D14),0)</f>
-        <v>104946.497289317</v>
+        <v>95405.9066266518</v>
       </c>
       <c r="J14" s="13"/>
       <c r="K14" s="28" t="n">
         <f aca="false">MAX(0,I14*TrancheA-J14)</f>
-        <v>73462.5481025219</v>
+        <v>66784.1346386563</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17878,7 +17878,7 @@
       </c>
       <c r="D15" s="36" t="n">
         <f aca="false">Disbursements!$C$14</f>
-        <v>69177.3093614383</v>
+        <v>109793.862368258</v>
       </c>
       <c r="E15" s="22" t="n">
         <v>367</v>
@@ -17897,12 +17897,12 @@
       </c>
       <c r="I15" s="28" t="n">
         <f aca="false">IFERROR(MIN(D15,E15/C15*D15),0)</f>
-        <v>27686.0114892561</v>
+        <v>43941.4912640683</v>
       </c>
       <c r="J15" s="13"/>
       <c r="K15" s="28" t="n">
         <f aca="false">MAX(0,I15*TrancheA-J15)</f>
-        <v>19380.2080424793</v>
+        <v>30759.0438848478</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17960,7 +17960,7 @@
       </c>
       <c r="D17" s="36" t="n">
         <f aca="false">Disbursements!$C$16</f>
-        <v>137225.741239892</v>
+        <v>124750.673854447</v>
       </c>
       <c r="E17" s="22" t="n">
         <v>1460</v>
@@ -17979,12 +17979,12 @@
       </c>
       <c r="I17" s="28" t="n">
         <f aca="false">IFERROR(MIN(D17,E17/C17*D17),0)</f>
-        <v>137225.741239892</v>
+        <v>124750.673854447</v>
       </c>
       <c r="J17" s="13"/>
       <c r="K17" s="28" t="n">
         <f aca="false">MAX(0,I17*TrancheA-J17)</f>
-        <v>96058.0188679245</v>
+        <v>87325.4716981132</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18001,7 +18001,7 @@
       </c>
       <c r="D18" s="36" t="n">
         <f aca="false">Disbursements!$C$17</f>
-        <v>122718.75</v>
+        <v>111562.5</v>
       </c>
       <c r="E18" s="22" t="n">
         <v>974</v>
@@ -18020,12 +18020,12 @@
       </c>
       <c r="I18" s="28" t="n">
         <f aca="false">IFERROR(MIN(D18,E18/C18*D18),0)</f>
-        <v>92086.3347457627</v>
+        <v>83714.8497688752</v>
       </c>
       <c r="J18" s="13"/>
       <c r="K18" s="28" t="n">
         <f aca="false">MAX(0,I18*TrancheA-J18)</f>
-        <v>64460.4343220339</v>
+        <v>58600.3948382126</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18083,7 +18083,7 @@
       </c>
       <c r="D20" s="36" t="n">
         <f aca="false">Disbursements!$C$19</f>
-        <v>39784.3839541547</v>
+        <v>36167.6217765043</v>
       </c>
       <c r="E20" s="22" t="n">
         <v>892</v>
@@ -18102,12 +18102,12 @@
       </c>
       <c r="I20" s="28" t="n">
         <f aca="false">IFERROR(MIN(D20,E20/C20*D20),0)</f>
-        <v>34997.7026500059</v>
+        <v>31816.0933181872</v>
       </c>
       <c r="J20" s="13"/>
       <c r="K20" s="28" t="n">
         <f aca="false">MAX(0,I20*TrancheA-J20)</f>
-        <v>24498.3918550042</v>
+        <v>22271.265322731</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18549,7 +18549,7 @@
       </c>
       <c r="D32" s="43" t="n">
         <f aca="false">SUM(D7:D31)</f>
-        <v>823387.761378275</v>
+        <v>753310.82158811</v>
       </c>
       <c r="E32" s="51" t="n">
         <f aca="false">SUM(E7:E31)</f>
@@ -18557,7 +18557,7 @@
       </c>
       <c r="I32" s="43" t="n">
         <f aca="false">SUM(I7:I31)</f>
-        <v>674279.66041605</v>
+        <v>602275.771011878</v>
       </c>
       <c r="J32" s="43" t="n">
         <f aca="false">SUM(J7:J31)</f>
@@ -18565,7 +18565,7 @@
       </c>
       <c r="K32" s="43" t="n">
         <f aca="false">SUM(K7:K31)</f>
-        <v>471995.762291235</v>
+        <v>421593.039708315</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18695,11 +18695,11 @@
       </c>
       <c r="I7" s="56" t="n">
         <f aca="false">IF(H7="",0,SUMIF(Pipeline!$C$7:$C$31,H7,'Eligibility &amp; Scoring'!$AK$7:$AK$31))</f>
-        <v>740750</v>
+        <v>510000</v>
       </c>
       <c r="J7" s="57" t="n">
         <f aca="false">IFERROR(I7/Envelope,0)</f>
-        <v>0.264081996434938</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18708,7 +18708,7 @@
       </c>
       <c r="C8" s="53" t="n">
         <f aca="false">Envelope</f>
-        <v>2805000</v>
+        <v>2550000</v>
       </c>
       <c r="E8" s="52" t="s">
         <v>255</v>
@@ -18723,7 +18723,7 @@
       </c>
       <c r="I8" s="56" t="n">
         <f aca="false">IF(H8="",0,SUMIF(Pipeline!$C$7:$C$31,H8,'Eligibility &amp; Scoring'!$AK$7:$AK$31))</f>
-        <v>1402500</v>
+        <v>1275000</v>
       </c>
       <c r="J8" s="57" t="n">
         <f aca="false">IFERROR(I8/Envelope,0)</f>
@@ -18736,7 +18736,7 @@
       </c>
       <c r="C9" s="53" t="n">
         <f aca="false">TotalRequested</f>
-        <v>3247750</v>
+        <v>2997500</v>
       </c>
       <c r="E9" s="52" t="s">
         <v>257</v>
@@ -18764,7 +18764,7 @@
       </c>
       <c r="C10" s="58" t="n">
         <f aca="false">IFERROR(TotalRequested/Envelope,0)</f>
-        <v>1.1578431372549</v>
+        <v>1.17549019607843</v>
       </c>
       <c r="E10" s="52" t="s">
         <v>259</v>
@@ -18779,11 +18779,11 @@
       </c>
       <c r="I10" s="56" t="n">
         <f aca="false">IF(H10="",0,SUMIF(Pipeline!$C$7:$C$31,H10,'Eligibility &amp; Scoring'!$AK$7:$AK$31))</f>
-        <v>661750</v>
+        <v>765000</v>
       </c>
       <c r="J10" s="57" t="n">
         <f aca="false">IFERROR(I10/Envelope,0)</f>
-        <v>0.235918003565062</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18792,7 +18792,7 @@
       </c>
       <c r="C11" s="53" t="n">
         <f aca="false">TotalAllocated</f>
-        <v>2805000</v>
+        <v>2550000</v>
       </c>
       <c r="E11" s="52" t="s">
         <v>260</v>
@@ -18820,14 +18820,14 @@
       </c>
       <c r="C12" s="53" t="n">
         <f aca="false">Disbursements!$C$31</f>
-        <v>823387.761378275</v>
+        <v>753310.82158811</v>
       </c>
       <c r="E12" s="52" t="s">
         <v>262</v>
       </c>
       <c r="F12" s="59" t="n">
         <f aca="false">IFERROR(SUMPRODUCT('Eligibility &amp; Scoring'!$AH$7:$AH$31,'Eligibility &amp; Scoring'!$AK$7:$AK$31)/TotalAllocated,0)</f>
-        <v>71.0248138720951</v>
+        <v>70.7439500329924</v>
       </c>
       <c r="H12" s="46" t="str">
         <f aca="false">IF('Fund Parameters'!$A$56="","",'Fund Parameters'!$A$56)</f>
@@ -18848,7 +18848,7 @@
       </c>
       <c r="C13" s="53" t="n">
         <f aca="false">Disbursements!$D$31</f>
-        <v>1981612.23862172</v>
+        <v>1796689.17841189</v>
       </c>
       <c r="H13" s="46" t="str">
         <f aca="false">IF('Fund Parameters'!$A$57="","",'Fund Parameters'!$A$57)</f>
@@ -18890,7 +18890,7 @@
       </c>
       <c r="C15" s="53" t="n">
         <f aca="false">TotalExpectedDisb</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
       <c r="H15" s="61" t="s">
         <v>266</v>
@@ -18910,14 +18910,14 @@
       </c>
       <c r="C16" s="53" t="n">
         <f aca="false">ExpectedDecommit</f>
-        <v>48552.9488986209</v>
+        <v>44616.6937595323</v>
       </c>
       <c r="H16" s="61" t="s">
         <v>267</v>
       </c>
       <c r="I16" s="48" t="n">
         <f aca="false">MAX(I7:I15)</f>
-        <v>1402500</v>
+        <v>1275000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18926,7 +18926,7 @@
       </c>
       <c r="C17" s="53" t="n">
         <f aca="false">MinCashBalance</f>
-        <v>-206447.051101379</v>
+        <v>44616.6937595322</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18935,7 +18935,7 @@
       </c>
       <c r="C18" s="58" t="n">
         <f aca="false">IFERROR(TotalAllocated/TotalExpectedDisb,0)</f>
-        <v>1.0176143230755</v>
+        <v>1.01780833042529</v>
       </c>
       <c r="H18" s="40" t="s">
         <v>270</v>
@@ -18970,15 +18970,15 @@
       </c>
       <c r="I20" s="62" t="n">
         <f aca="false">Disbursements!$G$31</f>
-        <v>156598.271110424</v>
+        <v>142362.06464584</v>
       </c>
       <c r="J20" s="62" t="n">
         <f aca="false">Disbursements!$G$60</f>
-        <v>876442.858615763</v>
+        <v>796766.235105239</v>
       </c>
       <c r="K20" s="62" t="n">
         <f aca="false">Disbursements!$G$94</f>
-        <v>1033041.12972619</v>
+        <v>939128.299751079</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18987,14 +18987,14 @@
       </c>
       <c r="C21" s="63" t="n">
         <f aca="false">SUMPRODUCT('Eligibility &amp; Scoring'!$C$7:$C$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>8010.03967761934</v>
+        <v>7960.3125</v>
       </c>
       <c r="E21" s="52" t="s">
         <v>278</v>
       </c>
       <c r="F21" s="53" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$N$7:$N$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>9753957.42922091</v>
+        <v>9645182.29166667</v>
       </c>
       <c r="H21" s="46" t="n">
         <f aca="false">FundStart-1+2</f>
@@ -19002,15 +19002,15 @@
       </c>
       <c r="I21" s="62" t="n">
         <f aca="false">Disbursements!$H$31</f>
-        <v>314245.030447853</v>
+        <v>287482.814784728</v>
       </c>
       <c r="J21" s="62" t="n">
         <f aca="false">Disbursements!$H$60</f>
-        <v>1105169.38000596</v>
+        <v>999922.943306651</v>
       </c>
       <c r="K21" s="62" t="n">
         <f aca="false">Disbursements!$H$94</f>
-        <v>2452455.54018</v>
+        <v>2226534.05784246</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19019,14 +19019,14 @@
       </c>
       <c r="C22" s="63" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$J$7:$J$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>6481.56643934697</v>
+        <v>6422.39583333333</v>
       </c>
       <c r="E22" s="52" t="s">
         <v>280</v>
       </c>
       <c r="F22" s="53" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$O$7:$O$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)+SUMPRODUCT(Pipeline!$P$7:$P$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>4392508.78280637</v>
+        <v>4322786.45833333</v>
       </c>
       <c r="H22" s="46" t="n">
         <f aca="false">FundStart-1+3</f>
@@ -19034,7 +19034,7 @@
       </c>
       <c r="I22" s="62" t="n">
         <f aca="false">Disbursements!$I$31</f>
-        <v>216429.380782786</v>
+        <v>198430.531594709</v>
       </c>
       <c r="J22" s="62" t="n">
         <f aca="false">Disbursements!$I$60</f>
@@ -19042,7 +19042,7 @@
       </c>
       <c r="K22" s="62" t="n">
         <f aca="false">Disbursements!$I$94</f>
-        <v>2668884.92096279</v>
+        <v>2424964.58943717</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19051,14 +19051,14 @@
       </c>
       <c r="C23" s="63" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$K$7:$K$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>650.16842322794</v>
+        <v>660.286458333333</v>
       </c>
       <c r="E23" s="52" t="s">
         <v>282</v>
       </c>
       <c r="F23" s="58" t="n">
         <f aca="false">IFERROR(PrivateMobilised/TotalAllocated,0)</f>
-        <v>1.56595678531421</v>
+        <v>1.69521037581699</v>
       </c>
       <c r="H23" s="46" t="n">
         <f aca="false">FundStart-1+4</f>
@@ -19066,7 +19066,7 @@
       </c>
       <c r="I23" s="62" t="n">
         <f aca="false">Disbursements!$J$31</f>
-        <v>75502.676557804</v>
+        <v>69326.6118717172</v>
       </c>
       <c r="J23" s="62" t="n">
         <f aca="false">Disbursements!$J$60</f>
@@ -19074,7 +19074,7 @@
       </c>
       <c r="K23" s="62" t="n">
         <f aca="false">Disbursements!$J$94</f>
-        <v>2744387.59752059</v>
+        <v>2494291.20130888</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19083,14 +19083,14 @@
       </c>
       <c r="C24" s="63" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$L$7:$L$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)+SUMPRODUCT(Pipeline!$M$7:$M$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>878.304815044431</v>
+        <v>877.630208333333</v>
       </c>
       <c r="E24" s="52" t="s">
         <v>284</v>
       </c>
       <c r="F24" s="58" t="n">
         <f aca="false">IFERROR(InvestMobilised/TotalAllocated,0)</f>
-        <v>3.4773466770841</v>
+        <v>3.78242442810458</v>
       </c>
       <c r="H24" s="46" t="n">
         <f aca="false">FundStart-1+5</f>
@@ -19098,7 +19098,7 @@
       </c>
       <c r="I24" s="62" t="n">
         <f aca="false">Disbursements!$K$31</f>
-        <v>12059.4535807879</v>
+        <v>11092.1049315831</v>
       </c>
       <c r="J24" s="62" t="n">
         <f aca="false">Disbursements!$K$60</f>
@@ -19106,7 +19106,7 @@
       </c>
       <c r="K24" s="62" t="n">
         <f aca="false">Disbursements!$K$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19115,14 +19115,14 @@
       </c>
       <c r="C25" s="63" t="n">
         <f aca="false">HHFunded*HHSize</f>
-        <v>32407.8321967349</v>
+        <v>32111.9791666667</v>
       </c>
       <c r="E25" s="52" t="s">
         <v>286</v>
       </c>
       <c r="F25" s="53" t="n">
         <f aca="false">IFERROR(TotalAllocated/ConnFunded,0)</f>
-        <v>350.185531269887</v>
+        <v>320.339182663997</v>
       </c>
       <c r="H25" s="46" t="n">
         <f aca="false">FundStart-1+6</f>
@@ -19138,7 +19138,7 @@
       </c>
       <c r="K25" s="62" t="n">
         <f aca="false">Disbursements!$L$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19147,14 +19147,14 @@
       </c>
       <c r="C26" s="63" t="n">
         <f aca="false">SUMPRODUCT(Pipeline!$T$7:$T$31,'Eligibility &amp; Scoring'!$AL$7:$AL$31)</f>
-        <v>50754.8873734243</v>
+        <v>50059.6354166667</v>
       </c>
       <c r="E26" s="52" t="s">
         <v>287</v>
       </c>
       <c r="F26" s="53" t="n">
         <f aca="false">IFERROR(TotalAllocated/PeopleFunded,0)</f>
-        <v>86.5531511941921</v>
+        <v>79.4096180358446</v>
       </c>
       <c r="H26" s="46" t="n">
         <f aca="false">FundStart-1+7</f>
@@ -19170,7 +19170,7 @@
       </c>
       <c r="K26" s="62" t="n">
         <f aca="false">Disbursements!$M$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19186,7 +19186,7 @@
       </c>
       <c r="F27" s="53" t="n">
         <f aca="false">IFERROR(TotalAllocated/CO2Funded,0)</f>
-        <v>55.2656137203592</v>
+        <v>50.9392443387834</v>
       </c>
       <c r="H27" s="46" t="n">
         <f aca="false">FundStart-1+8</f>
@@ -19202,7 +19202,7 @@
       </c>
       <c r="K27" s="62" t="n">
         <f aca="false">Disbursements!$N$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19220,7 +19220,7 @@
       </c>
       <c r="K28" s="62" t="n">
         <f aca="false">Disbursements!$O$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="K29" s="62" t="n">
         <f aca="false">Disbursements!$P$94</f>
-        <v>2756447.05110138</v>
+        <v>2505383.30624047</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19260,7 +19260,7 @@
       </c>
       <c r="C31" s="60" t="n">
         <f aca="false">IFERROR((TotalExpectedDisb-AllocGrant)/AllocRBF,0)</f>
-        <v>0.94103270515298</v>
+        <v>0.940772530433755</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19311,7 +19311,7 @@
       </c>
       <c r="C38" s="65" t="str">
         <f aca="false">IF(MinCashBalance&gt;=0,"YES","NO - reduce over-commitment")</f>
-        <v>NO - reduce over-commitment</v>
+        <v>YES</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>